<commit_message>
Atualizacao de arquivos - 05/08/2026 17:05:44,40
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/NPS Franquias/nps-franquias/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="383" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9F7506C-0E86-4557-BACF-E1FFEFB99F88}"/>
+  <xr:revisionPtr revIDLastSave="493" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09789F30-026A-4D33-8660-E3A83D510FDD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11314" uniqueCount="1586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11456" uniqueCount="1618">
   <si>
     <t>ID</t>
   </si>
@@ -4953,12 +4953,113 @@
   <si>
     <t>O técnico foi fazer a manutenção semestral e deixou o filtro com um barulho ensurdecedor.</t>
   </si>
+  <si>
+    <t>SEMPRE DIFICULDADES DE TROCA DO FILTRO A CADA 6 MESES VCS SÓ TROCAM A CADA ANO E NÃO CONCORDAMOS. NESSA ÚLTIMA VEZ NÃO RECEBI AVISO DA VISITA DA MANUNTENÇÃO E TIVERAM MUITA SORTE QUE HAVIA GENTE NO APARTAMENTO.E FIZERAM A MANUTENÇÃO SEM A PRESENÇA DO RESPONSÁVEL.</t>
+  </si>
+  <si>
+    <t>Esse serviço de atendimento de máquina é horrível, a máquina está programada para o benefício da BRASTEMP, não existe outro canal além de pessoas ligarem em nome da brastemp para cobrança. Serviço anti profissional, sem transparência e irritante. Marcam visitas e o técnico não aparece, você se indispoe com esse serviço confuso e nada prático. Está pior do que antes, penso até de encerrar o contrato.</t>
+  </si>
+  <si>
+    <t>Meu purificador continua com o gotejamento do qual eu havia reclamado, o técnico não fez nada para consertar...</t>
+  </si>
+  <si>
+    <t>PÉSSIMO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não tem atendimento, mais fácil falar com o papa do que falar com vocês </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Pela primeira vez vocês chegaram dentro da hora marcada.
+   Porém quando entrei em contato pedi um concerto, falei o que estava acontecendo e a empresa esqueceu de me falar que eu teria que desligar da tomada com 24 hs de antecedência, final nao puderam fazer o serviço. 
+   É lamentável </t>
+  </si>
+  <si>
+    <t>Na sexta dia 31, o tecnico veio para constar o defeito no aparelho e marcamos para terça dia 4/08 MANHA para a troca da peça, hoje recebi a mensagem para confirmar para dia 4/08 tarde. Não foi o combinado e depois de passar um tempao no telefone para conseguir um atendimento não virtual, a atendente não fez nenhum esforço para eu poder reestabelecer o meu agendamento que fizemos na sexta com o tecnico ou seja dia 4/08 MANHA. A unica solução foi aceitar o agendamento TARDE senão, o conserto ia para outra semana. Estou sem agua gelada já faz muito tempo e acho absurdo essa dificuldade para consertar. Pensando em trocar de fornecedor. O atendimento da Brastemp é péssimo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solicitei a instalação de um pressurizador, assim que o técnico foi embora o meu bebedor começou a vazar água, já vieram dois técnicos e o problema não foi resolvido, já estou agendando mais uma visita. Esse é o meu problema com a Culligan no momento.
+</t>
+  </si>
+  <si>
+    <t>Entrei para solicitar a troca de titularidade e fui informada que levará 45 dias para formalizar. Solicitei então a fatura, pois o débito automático foi descadastrado sem motivo e sem aviso, informaram que não tinham acesso e que terei que ligar novamente no dia do vencimento para solicitar. 40 minutos para isso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desisti do serviço. Muitos chamados não atendidos, queixas repetidas. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">O Tecnico não apareceu como sempre
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A pessoa que veio aqui não deixou documento com data de revisão, e não trocou o filtro. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipamento mal instalado. Ficou vazando água. Não funciona corretamente na função gaseificada. Péssimo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">porque deixou o filtro com botao ruim
+</t>
+  </si>
+  <si>
+    <t>Motivo</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>"péssimo" sem motivo específico</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>impossível contato, sem atendimento</t>
+  </si>
+  <si>
+    <t>esqueceram de avisar desligar tomada 24h</t>
+  </si>
+  <si>
+    <t>agendamento alterado + atendente não ajudou + sem água gelada</t>
+  </si>
+  <si>
+    <t>REVISAR</t>
+  </si>
+  <si>
+    <t>bebedouro vazou após visita + reincidência (R5)</t>
+  </si>
+  <si>
+    <t>troca filtro 6/6 meses não feita + sem aviso (R10)</t>
+  </si>
+  <si>
+    <t>atendimento não resolve, 40 min</t>
+  </si>
+  <si>
+    <t>chamados não atendidos, queixas repetidas (R10)</t>
+  </si>
+  <si>
+    <t>técnico não apareceu (R8)</t>
+  </si>
+  <si>
+    <t>sem comprovante + não trocou filtro (R3)</t>
+  </si>
+  <si>
+    <t>atendimento robotizado ruim + técnico não aparece</t>
+  </si>
+  <si>
+    <t>mal instalado, vazando + não gaseifica (R5)</t>
+  </si>
+  <si>
+    <t>filtro com botão ruim após serviço</t>
+  </si>
+  <si>
+    <t>gotejamento persiste, técnico não consertou (R10)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4972,16 +5073,29 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -5004,11 +5118,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5024,6 +5149,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5325,9 +5456,31 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="8">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{A99F678C-0A58-4B38-BD6D-52FA45E08A1C}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;779238cc-993e-4694-81ed-dd28055a6f94&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1414"/>
+  <dimension ref="A1:M1428"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -5344,7 +5497,7 @@
     <col min="12" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -5378,8 +5531,14 @@
       <c r="K1" s="4" t="s">
         <v>1438</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="4" t="s">
+        <v>1600</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>1601</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -5414,7 +5573,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -5449,7 +5608,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -5484,7 +5643,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -5519,7 +5678,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -5554,7 +5713,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -5589,7 +5748,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -5624,7 +5783,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -5659,7 +5818,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -5694,7 +5853,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -5729,7 +5888,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -5764,7 +5923,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -5799,7 +5958,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -5834,7 +5993,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -5869,7 +6028,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -54621,7 +54780,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1409" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+    <row r="1409" spans="1:13" ht="165" x14ac:dyDescent="0.25">
       <c r="A1409" s="4">
         <v>413</v>
       </c>
@@ -54656,7 +54815,7 @@
         <v>1463</v>
       </c>
     </row>
-    <row r="1410" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1410" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1410" s="4">
         <v>414</v>
       </c>
@@ -54691,7 +54850,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1411" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1411" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1411" s="4">
         <v>415</v>
       </c>
@@ -54726,7 +54885,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1412" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1412" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1412" s="4">
         <v>416</v>
       </c>
@@ -54761,7 +54920,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1413" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1413" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1413" s="4">
         <v>417</v>
       </c>
@@ -54796,7 +54955,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1414" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1414" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1414" s="4">
         <v>418</v>
       </c>
@@ -54831,7 +54990,582 @@
         <v>1441</v>
       </c>
     </row>
+    <row r="1415" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1415" s="4">
+        <v>419</v>
+      </c>
+      <c r="B1415" s="6" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1415" s="4">
+        <v>93363</v>
+      </c>
+      <c r="D1415" s="2">
+        <v>46237.667943263892</v>
+      </c>
+      <c r="E1415" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1415" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1415" s="4" t="s">
+        <v>1589</v>
+      </c>
+      <c r="H1415" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1415" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1415" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1415" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1415" s="4" t="s">
+        <v>1602</v>
+      </c>
+      <c r="M1415" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1416" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1416" s="4">
+        <v>420</v>
+      </c>
+      <c r="B1416" s="6" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1416" s="4">
+        <v>108557</v>
+      </c>
+      <c r="D1416" s="2">
+        <v>46237.680220752314</v>
+      </c>
+      <c r="E1416" s="6" t="s">
+        <v>1430</v>
+      </c>
+      <c r="F1416" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1416" s="4" t="s">
+        <v>1590</v>
+      </c>
+      <c r="H1416" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1416" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="J1416" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1416" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1416" s="4" t="s">
+        <v>1604</v>
+      </c>
+      <c r="M1416" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1417" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1417" s="4">
+        <v>421</v>
+      </c>
+      <c r="B1417" s="6" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1417" s="4">
+        <v>105311</v>
+      </c>
+      <c r="D1417" s="2">
+        <v>46237.693124479163</v>
+      </c>
+      <c r="E1417" s="6" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1417" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1417" s="4" t="s">
+        <v>1591</v>
+      </c>
+      <c r="H1417" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1417" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1417" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1417" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1417" s="4" t="s">
+        <v>1605</v>
+      </c>
+      <c r="M1417" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1418" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1418" s="4">
+        <v>422</v>
+      </c>
+      <c r="B1418" s="7" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1418" s="4">
+        <v>104155</v>
+      </c>
+      <c r="D1418" s="2">
+        <v>46237.922759918984</v>
+      </c>
+      <c r="E1418" s="7" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1418" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1418" s="4" t="s">
+        <v>1592</v>
+      </c>
+      <c r="H1418" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1418" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1418" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1418" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1418" s="4" t="s">
+        <v>1606</v>
+      </c>
+      <c r="M1418" s="4" t="s">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="1419" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1419" s="4">
+        <v>423</v>
+      </c>
+      <c r="B1419" s="6" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1419" s="4">
+        <v>112676</v>
+      </c>
+      <c r="D1419" s="2">
+        <v>46237.985251817132</v>
+      </c>
+      <c r="E1419" s="6" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1419" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1419" s="4" t="s">
+        <v>1593</v>
+      </c>
+      <c r="H1419" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1419" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1419" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1419" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1419" s="4" t="s">
+        <v>1608</v>
+      </c>
+      <c r="M1419" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1420" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1420" s="4">
+        <v>424</v>
+      </c>
+      <c r="B1420" s="7" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1420" s="4">
+        <v>98227</v>
+      </c>
+      <c r="D1420" s="2">
+        <v>46237.994408136576</v>
+      </c>
+      <c r="E1420" s="7" t="s">
+        <v>1484</v>
+      </c>
+      <c r="F1420" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1420" s="4" t="s">
+        <v>1586</v>
+      </c>
+      <c r="H1420" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1420" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1420" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1420" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1420" s="4" t="s">
+        <v>1609</v>
+      </c>
+      <c r="M1420" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1421" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1421" s="4">
+        <v>425</v>
+      </c>
+      <c r="B1421" s="6" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1421" s="4">
+        <v>105177</v>
+      </c>
+      <c r="D1421" s="2">
+        <v>46238.55375561343</v>
+      </c>
+      <c r="E1421" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1421" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1421" s="4" t="s">
+        <v>1594</v>
+      </c>
+      <c r="H1421" s="4" t="s">
+        <v>1534</v>
+      </c>
+      <c r="I1421" s="4" t="s">
+        <v>1561</v>
+      </c>
+      <c r="J1421" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1421" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1421" s="4" t="s">
+        <v>1610</v>
+      </c>
+      <c r="M1421" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1422" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1422" s="4">
+        <v>426</v>
+      </c>
+      <c r="B1422" s="7" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1422" s="4">
+        <v>101549</v>
+      </c>
+      <c r="D1422" s="2">
+        <v>46238.658281145836</v>
+      </c>
+      <c r="E1422" s="7" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1422" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1422" s="4" t="s">
+        <v>1595</v>
+      </c>
+      <c r="H1422" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1422" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1422" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1422" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1422" s="4" t="s">
+        <v>1611</v>
+      </c>
+      <c r="M1422" s="4" t="s">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="1423" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1423" s="4">
+        <v>427</v>
+      </c>
+      <c r="B1423" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1423" s="4">
+        <v>95266</v>
+      </c>
+      <c r="D1423" s="2">
+        <v>46238.74402096065</v>
+      </c>
+      <c r="E1423" s="4" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1423" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1423" s="4" t="s">
+        <v>1596</v>
+      </c>
+      <c r="H1423" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1423" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1423" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1423" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1423" s="4" t="s">
+        <v>1612</v>
+      </c>
+      <c r="M1423" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1424" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1424" s="4">
+        <v>428</v>
+      </c>
+      <c r="B1424" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1424" s="4">
+        <v>95186</v>
+      </c>
+      <c r="D1424" s="2">
+        <v>46238.750557662039</v>
+      </c>
+      <c r="E1424" s="4" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1424" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1424" s="4" t="s">
+        <v>1597</v>
+      </c>
+      <c r="H1424" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1424" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1424" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1424" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1424" s="4" t="s">
+        <v>1613</v>
+      </c>
+      <c r="M1424" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1425" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1425" s="4">
+        <v>429</v>
+      </c>
+      <c r="B1425" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1425" s="4">
+        <v>104439</v>
+      </c>
+      <c r="D1425" s="2">
+        <v>46239.074787708334</v>
+      </c>
+      <c r="E1425" s="4" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1425" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1425" s="4" t="s">
+        <v>1587</v>
+      </c>
+      <c r="H1425" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1425" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1425" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1425" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1425" s="4" t="s">
+        <v>1614</v>
+      </c>
+      <c r="M1425" s="4" t="s">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="1426" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1426" s="4">
+        <v>430</v>
+      </c>
+      <c r="B1426" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1426" s="4">
+        <v>88461</v>
+      </c>
+      <c r="D1426" s="2">
+        <v>46239.552590254629</v>
+      </c>
+      <c r="E1426" s="4" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1426" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1426" s="4" t="s">
+        <v>1598</v>
+      </c>
+      <c r="H1426" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1426" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1426" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1426" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1426" s="4" t="s">
+        <v>1615</v>
+      </c>
+      <c r="M1426" s="4" t="s">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="1427" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1427" s="4">
+        <v>431</v>
+      </c>
+      <c r="B1427" s="4" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1427" s="4">
+        <v>103851</v>
+      </c>
+      <c r="D1427" s="2">
+        <v>46239.637758738427</v>
+      </c>
+      <c r="E1427" s="4" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1427" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1427" s="4" t="s">
+        <v>1599</v>
+      </c>
+      <c r="H1427" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1427" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1427" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1427" s="4" t="s">
+        <v>1442</v>
+      </c>
+      <c r="L1427" s="4" t="s">
+        <v>1616</v>
+      </c>
+      <c r="M1427" s="4" t="s">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="1428" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1428" s="4">
+        <v>432</v>
+      </c>
+      <c r="B1428" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1428" s="4">
+        <v>109246</v>
+      </c>
+      <c r="D1428" s="2">
+        <v>46239.658815532406</v>
+      </c>
+      <c r="E1428" s="4" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1428" s="4" t="s">
+        <v>1464</v>
+      </c>
+      <c r="G1428" s="4" t="s">
+        <v>1588</v>
+      </c>
+      <c r="H1428" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1428" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1428" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1428" s="4" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1428" s="4" t="s">
+        <v>1617</v>
+      </c>
+      <c r="M1428" s="4" t="s">
+        <v>1603</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualizacao de arquivos - 06/08/2026 10:07:08,06
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="493" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09789F30-026A-4D33-8660-E3A83D510FDD}"/>
+  <xr:revisionPtr revIDLastSave="507" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED1B5784-40C2-4465-AEE7-3CA41A033BC2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11456" uniqueCount="1618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11434" uniqueCount="1601">
   <si>
     <t>ID</t>
   </si>
@@ -5001,58 +5001,7 @@
 </t>
   </si>
   <si>
-    <t>Motivo</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>"péssimo" sem motivo específico</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>impossível contato, sem atendimento</t>
-  </si>
-  <si>
-    <t>esqueceram de avisar desligar tomada 24h</t>
-  </si>
-  <si>
-    <t>agendamento alterado + atendente não ajudou + sem água gelada</t>
-  </si>
-  <si>
-    <t>REVISAR</t>
-  </si>
-  <si>
-    <t>bebedouro vazou após visita + reincidência (R5)</t>
-  </si>
-  <si>
-    <t>troca filtro 6/6 meses não feita + sem aviso (R10)</t>
-  </si>
-  <si>
-    <t>atendimento não resolve, 40 min</t>
-  </si>
-  <si>
-    <t>chamados não atendidos, queixas repetidas (R10)</t>
-  </si>
-  <si>
-    <t>técnico não apareceu (R8)</t>
-  </si>
-  <si>
-    <t>sem comprovante + não trocou filtro (R3)</t>
-  </si>
-  <si>
-    <t>atendimento robotizado ruim + técnico não aparece</t>
-  </si>
-  <si>
-    <t>mal instalado, vazando + não gaseifica (R5)</t>
-  </si>
-  <si>
-    <t>filtro com botão ruim após serviço</t>
-  </si>
-  <si>
-    <t>gotejamento persiste, técnico não consertou (R10)</t>
+    <t xml:space="preserve">Pq a Culligan me passou informaçoes indevidas ref, numero do caso e numero OS, por várias vezes que o técnico veio para fazer o servico, e nao batia as informaçoes. Inclusive no dia 04/08/26 o técnico só subiu, pq o zelador o acompanhou e ficou junto enqto ele fazia o serviço, e eu fiquei fora do apto rezando p/ que nao fosse um ladrao! ISSO É UM ABSURDO!!!! </t>
   </si>
 </sst>
 </file>
@@ -5480,7 +5429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1428"/>
+  <dimension ref="A1:K1429"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -5497,7 +5446,7 @@
     <col min="12" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -5531,14 +5480,8 @@
       <c r="K1" s="4" t="s">
         <v>1438</v>
       </c>
-      <c r="L1" s="4" t="s">
-        <v>1600</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>1601</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -5573,7 +5516,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -5608,7 +5551,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -5643,7 +5586,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -5678,7 +5621,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -5713,7 +5656,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -5748,7 +5691,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -5783,7 +5726,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -5818,7 +5761,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -5853,7 +5796,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -5888,7 +5831,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -5923,7 +5866,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -5958,7 +5901,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -5993,7 +5936,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -6028,7 +5971,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -54780,7 +54723,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1409" spans="1:13" ht="165" x14ac:dyDescent="0.25">
+    <row r="1409" spans="1:11" ht="165" x14ac:dyDescent="0.25">
       <c r="A1409" s="4">
         <v>413</v>
       </c>
@@ -54815,7 +54758,7 @@
         <v>1463</v>
       </c>
     </row>
-    <row r="1410" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1410" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1410" s="4">
         <v>414</v>
       </c>
@@ -54850,7 +54793,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1411" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1411" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1411" s="4">
         <v>415</v>
       </c>
@@ -54885,7 +54828,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1412" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1412" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1412" s="4">
         <v>416</v>
       </c>
@@ -54920,7 +54863,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1413" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1413" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1413" s="4">
         <v>417</v>
       </c>
@@ -54955,7 +54898,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1414" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1414" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1414" s="4">
         <v>418</v>
       </c>
@@ -54990,7 +54933,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="1415" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1415" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1415" s="4">
         <v>419</v>
       </c>
@@ -55024,14 +54967,8 @@
       <c r="K1415" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1415" s="4" t="s">
-        <v>1602</v>
-      </c>
-      <c r="M1415" s="4" t="s">
-        <v>1603</v>
-      </c>
-    </row>
-    <row r="1416" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1416" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1416" s="4">
         <v>420</v>
       </c>
@@ -55065,14 +55002,8 @@
       <c r="K1416" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1416" s="4" t="s">
-        <v>1604</v>
-      </c>
-      <c r="M1416" s="4" t="s">
-        <v>1603</v>
-      </c>
-    </row>
-    <row r="1417" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1417" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1417" s="4">
         <v>421</v>
       </c>
@@ -55106,14 +55037,8 @@
       <c r="K1417" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1417" s="4" t="s">
-        <v>1605</v>
-      </c>
-      <c r="M1417" s="4" t="s">
-        <v>1603</v>
-      </c>
-    </row>
-    <row r="1418" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1418" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1418" s="4">
         <v>422</v>
       </c>
@@ -55147,14 +55072,8 @@
       <c r="K1418" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1418" s="4" t="s">
-        <v>1606</v>
-      </c>
-      <c r="M1418" s="4" t="s">
-        <v>1607</v>
-      </c>
-    </row>
-    <row r="1419" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1419" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1419" s="4">
         <v>423</v>
       </c>
@@ -55188,14 +55107,8 @@
       <c r="K1419" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1419" s="4" t="s">
-        <v>1608</v>
-      </c>
-      <c r="M1419" s="4" t="s">
-        <v>1603</v>
-      </c>
-    </row>
-    <row r="1420" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1420" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1420" s="4">
         <v>424</v>
       </c>
@@ -55229,14 +55142,8 @@
       <c r="K1420" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1420" s="4" t="s">
-        <v>1609</v>
-      </c>
-      <c r="M1420" s="4" t="s">
-        <v>1603</v>
-      </c>
-    </row>
-    <row r="1421" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1421" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1421" s="4">
         <v>425</v>
       </c>
@@ -55270,14 +55177,8 @@
       <c r="K1421" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1421" s="4" t="s">
-        <v>1610</v>
-      </c>
-      <c r="M1421" s="4" t="s">
-        <v>1603</v>
-      </c>
-    </row>
-    <row r="1422" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1422" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1422" s="4">
         <v>426</v>
       </c>
@@ -55311,14 +55212,8 @@
       <c r="K1422" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1422" s="4" t="s">
-        <v>1611</v>
-      </c>
-      <c r="M1422" s="4" t="s">
-        <v>1607</v>
-      </c>
-    </row>
-    <row r="1423" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1423" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1423" s="4">
         <v>427</v>
       </c>
@@ -55352,14 +55247,8 @@
       <c r="K1423" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1423" s="4" t="s">
-        <v>1612</v>
-      </c>
-      <c r="M1423" s="4" t="s">
-        <v>1603</v>
-      </c>
-    </row>
-    <row r="1424" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1424" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1424" s="4">
         <v>428</v>
       </c>
@@ -55393,14 +55282,8 @@
       <c r="K1424" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1424" s="4" t="s">
-        <v>1613</v>
-      </c>
-      <c r="M1424" s="4" t="s">
-        <v>1603</v>
-      </c>
-    </row>
-    <row r="1425" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1425" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1425" s="4">
         <v>429</v>
       </c>
@@ -55434,14 +55317,8 @@
       <c r="K1425" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1425" s="4" t="s">
-        <v>1614</v>
-      </c>
-      <c r="M1425" s="4" t="s">
-        <v>1607</v>
-      </c>
-    </row>
-    <row r="1426" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1426" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1426" s="4">
         <v>430</v>
       </c>
@@ -55475,14 +55352,8 @@
       <c r="K1426" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1426" s="4" t="s">
-        <v>1615</v>
-      </c>
-      <c r="M1426" s="4" t="s">
-        <v>1607</v>
-      </c>
-    </row>
-    <row r="1427" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1427" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1427" s="4">
         <v>431</v>
       </c>
@@ -55516,14 +55387,8 @@
       <c r="K1427" s="4" t="s">
         <v>1442</v>
       </c>
-      <c r="L1427" s="4" t="s">
-        <v>1616</v>
-      </c>
-      <c r="M1427" s="4" t="s">
-        <v>1607</v>
-      </c>
-    </row>
-    <row r="1428" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1428" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1428" s="4">
         <v>432</v>
       </c>
@@ -55557,11 +55422,40 @@
       <c r="K1428" s="4" t="s">
         <v>1440</v>
       </c>
-      <c r="L1428" s="4" t="s">
-        <v>1617</v>
-      </c>
-      <c r="M1428" s="4" t="s">
-        <v>1603</v>
+    </row>
+    <row r="1429" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1429" s="4">
+        <v>433</v>
+      </c>
+      <c r="B1429" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1429">
+        <v>104833</v>
+      </c>
+      <c r="D1429" s="2">
+        <v>46239.658815532406</v>
+      </c>
+      <c r="E1429" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1429" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1429" t="s">
+        <v>1600</v>
+      </c>
+      <c r="H1429" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1429" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1429" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1429" s="4" t="s">
+        <v>1440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 07/08/2026  9:07:29,09
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="507" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED1B5784-40C2-4465-AEE7-3CA41A033BC2}"/>
+  <xr:revisionPtr revIDLastSave="532" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95E3DBA3-F6BA-4ADD-9D72-7EB751D62698}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-2580" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11434" uniqueCount="1601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11498" uniqueCount="1610">
   <si>
     <t>ID</t>
   </si>
@@ -5002,6 +5002,42 @@
   </si>
   <si>
     <t xml:space="preserve">Pq a Culligan me passou informaçoes indevidas ref, numero do caso e numero OS, por várias vezes que o técnico veio para fazer o servico, e nao batia as informaçoes. Inclusive no dia 04/08/26 o técnico só subiu, pq o zelador o acompanhou e ficou junto enqto ele fazia o serviço, e eu fiquei fora do apto rezando p/ que nao fosse um ladrao! ISSO É UM ABSURDO!!!! </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Havia agendado entre 08:00 e 13:00… fiquei esperando até 13:12 
+Cancelei porque tinha que sair….. 
+para minha supresa quando voltei para casa às 14:00 soube que o técnico veio e quem teve de atender foi minha esposa que estava acamada…..vergonha f de o atendimento, que piorou muito depois da união Brastemp-Culligan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Embora instalação tenha sido realizada.
+O grande problema ocorreu entre a equipe de agendamento e instalação, aguardamos 2 sábados, dia permitido para instalação e mesmo com a confirmação de agendamento, o técnico não compareceu, por se tratar de dia que o escritório fecha, causou mais transtorno. Tivemos que convocar um funcionário somente para receber o técnico e ficou aguardando todo o período de 8h00 as 13h00, tempo e dinheiro perdido.
+Durante a semana, ficavam tentando ir instalar, sem agendamento, mesmo sendo informado que não seria permitido. Bem Desorganizado.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque achei que o filtro seria trocado de 6 em 6 meses, pra ter valido a pena eu ter assinado o serviço.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico não atendeu o que precisava ser feito, e empresa demora muito para agendar uma simples troca de filtro que já tinha passado do prazo de troca </t>
+  </si>
+  <si>
+    <t>Tudo nessa empresa é demorado. Vou cancelar o meu contrato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prestador serviço  de  nome  Caique  Ribeiro não  fez  teste  na  água, preciso trocar meu aparelho  desde que assinei o contrato está com problemas no botão da saída de água. 
+já foi  feito  diversos  reparos  em todas as manutenção  e  nunca  resolve,  e  simplesmente o técnico disse  que  era  mais  fácil eu  cancelar a  assinatura  porque  dava  muito  trabalho para  ele  fazer a  troca,  tinha  que  filmar  o  problema  em  fim,  para  eu  cancelar e  depois pedir  de  novo  acredita ,  para  não  ter  trabalho. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">fiquei impressionado com a velocidade que o prestador de serviço, Erivan Luciano da Silva entrou e saiu condomínio, e ainda fez a manutenção, 15 minutos, e pedindo esclarecimentos através do telefone 11 98699-7958 sobre o procedimento de atendimento, a atendente Layane, pouco se interessou em ouvir minha reclamação, mandando eu aguardar o protocolo 00264921.
+Conforme for o laudo que eu receber, irei procurar maiores esclarecimentos através do Jurídico.
+</t>
+  </si>
+  <si>
+    <t>Horrível, muito tempo esperando a manutenção em um bebedouro com a agua amarela.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo </t>
   </si>
 </sst>
 </file>
@@ -5082,7 +5118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5104,6 +5140,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5429,7 +5468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1429"/>
+  <dimension ref="A1:K1437"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -55458,6 +55497,286 @@
         <v>1440</v>
       </c>
     </row>
+    <row r="1430" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1430" s="4">
+        <v>434</v>
+      </c>
+      <c r="B1430" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1430" s="8">
+        <v>103626</v>
+      </c>
+      <c r="D1430" s="2">
+        <v>46240.428025729168</v>
+      </c>
+      <c r="E1430" s="8" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1430" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1430" s="8" t="s">
+        <v>1601</v>
+      </c>
+      <c r="H1430" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1430" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1430" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1430" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1431" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1431" s="4">
+        <v>435</v>
+      </c>
+      <c r="B1431" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1431" s="8">
+        <v>110309</v>
+      </c>
+      <c r="D1431" s="2">
+        <v>46240.522614340283</v>
+      </c>
+      <c r="E1431" s="8" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1431" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1431" s="8" t="s">
+        <v>1602</v>
+      </c>
+      <c r="H1431" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1431" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1431" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1431" s="8" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1432" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1432" s="4">
+        <v>436</v>
+      </c>
+      <c r="B1432" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1432" s="8">
+        <v>114401</v>
+      </c>
+      <c r="D1432" s="2">
+        <v>46240.554278495372</v>
+      </c>
+      <c r="E1432" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1432" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1432" s="8" t="s">
+        <v>1603</v>
+      </c>
+      <c r="H1432" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1432" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1432" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1432" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1433" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1433" s="4">
+        <v>437</v>
+      </c>
+      <c r="B1433" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1433" s="8">
+        <v>112740</v>
+      </c>
+      <c r="D1433" s="2">
+        <v>46240.566327060187</v>
+      </c>
+      <c r="E1433" s="8" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1433" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1433" s="8" t="s">
+        <v>1604</v>
+      </c>
+      <c r="H1433" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1433" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1433" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1433" s="8" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1434" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1434" s="4">
+        <v>438</v>
+      </c>
+      <c r="B1434" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1434" s="8">
+        <v>98452</v>
+      </c>
+      <c r="D1434" s="2">
+        <v>46240.703195682872</v>
+      </c>
+      <c r="E1434" s="8" t="s">
+        <v>1508</v>
+      </c>
+      <c r="F1434" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1434" s="8" t="s">
+        <v>1605</v>
+      </c>
+      <c r="H1434" s="4" t="s">
+        <v>1609</v>
+      </c>
+      <c r="I1434" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1434" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1434" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1435" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1435" s="4">
+        <v>439</v>
+      </c>
+      <c r="B1435" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1435" s="8">
+        <v>110003</v>
+      </c>
+      <c r="D1435" s="2">
+        <v>46240.721779143518</v>
+      </c>
+      <c r="E1435" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1435" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1435" s="8" t="s">
+        <v>1606</v>
+      </c>
+      <c r="H1435" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1435" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1435" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1435" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1436" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1436" s="4">
+        <v>440</v>
+      </c>
+      <c r="B1436" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1436" s="8">
+        <v>89116</v>
+      </c>
+      <c r="D1436" s="2">
+        <v>46240.751161192129</v>
+      </c>
+      <c r="E1436" s="8" t="s">
+        <v>1430</v>
+      </c>
+      <c r="F1436" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1436" s="8" t="s">
+        <v>1607</v>
+      </c>
+      <c r="H1436" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1436" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1436" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1436" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1437" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1437" s="4">
+        <v>441</v>
+      </c>
+      <c r="B1437" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1437" s="8">
+        <v>113608</v>
+      </c>
+      <c r="D1437" s="2">
+        <v>46240.822670208327</v>
+      </c>
+      <c r="E1437" s="8" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1437" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1437" s="8" t="s">
+        <v>1608</v>
+      </c>
+      <c r="H1437" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1437" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1437" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1437" s="8" t="s">
+        <v>1463</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 11/08/2026 11:22:04,12
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="532" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95E3DBA3-F6BA-4ADD-9D72-7EB751D62698}"/>
+  <xr:revisionPtr revIDLastSave="616" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BEBF561-D19C-459A-89D6-5A7D18CDF1B6}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-2580" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23880" yWindow="1920" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1414</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1450</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11498" uniqueCount="1610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11630" uniqueCount="1644">
   <si>
     <t>ID</t>
   </si>
@@ -5039,12 +5039,128 @@
   <si>
     <t xml:space="preserve">Campo </t>
   </si>
+  <si>
+    <t>FRQ CAMPINAS R02</t>
+  </si>
+  <si>
+    <t>FRQ RECIFE PE R02</t>
+  </si>
+  <si>
+    <t>AT NATAL RN R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>FRQ SJCAMPOS SP R02 - MATRIZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Não fez o que precisava. Chega sempre no horário de almoço que foi pedido para eu acompanhar , não faz o combinado nunca com o cliente. Insatisfeito. /// e esta demorando para instalar o outro equipamento que tenho .. isso porque sou cliente a muito tempo e tenho 05 purificadores.  </t>
+  </si>
+  <si>
+    <t>O aparelho foi consertado mas achei que diante da extrema necessidade demorar 4 dias para atender foi muito já que se trata de agua para beber. Mas o funcionário foi excelente e consertou o defeito quando esteve aqui.</t>
+  </si>
+  <si>
+    <t>Minha insatisfação com empresa Brastemp e Culligan é gigante!
+Se eu fosse citar todos os.problemas que eu estou tendo esse espaço aqui tá pequeno.
+E de verdade essa pesquisa, não passe de uma mentira porque nem a reclamação que eu fiz no site RECLAME AQUI, a empresa se importou. 
+Vocês simplesmente ignora nossas reclamações, atendentes(humanos) despreparados, não te dão devolutiva de um protocolo quando dão , não sabe nem do que se trata.
+É uma falta de respeito e olha que eu tinha 3 FILTROS, estou CANCELANDO TODOS e com certeza meu marketing será NEGATIVO.</t>
+  </si>
+  <si>
+    <t>DE ACORDO COM MINHA SOLICITAÇÃO VEIO UM TÉCNICO NO ÚLTIMO DIA 06 DE AGOSTO. NÃO TERMINOU O SERVIÇO E FICOU , EM PRINCÍPIO, QUE SERIA CONCLUÍDO O REPARO EM 48 HS. NO DIA 08 FIQUEI ESPERANDO A VINDA DE UM TÉCNICO. COMO ESTAVA FICANDO TARDE, LIGUEI PARA A BRASTEMP E FUI INFORMADO DE QUE HAVIA UM AGENDAMENTO PARA VISITA TÉCNICA PARA O DIA 25. CONSEGUI COM A ATENDENTE MUDAR PARA O PRÓXIMO DIA 11. ESPERA QUE O SERVIÇO SEJA CONCLUÍDO, ENTÃO.</t>
+  </si>
+  <si>
+    <t>Pois marcamos a troca de dois elementos filtrantes, pois temos 02 contratos e a troca do botão de um deles de liga e desliga. O funcionário foi excelente ,mas fiz a marcação por telefone e sempre agendam errado.
+Estou no aguardo para a troca do elemento filtrante e do botão de liga e desliga. Urgente</t>
+  </si>
+  <si>
+    <t>Agendaram uma visita técnica para troca do filtro do purificador e NÃO CUMPRIRAM, remarcando para mais de uma semana, apesar dos meus argumentos de que estávamos sem usar o purificador.</t>
+  </si>
+  <si>
+    <t>Boa tarde.
+Já solicitei diversas vezes o conserto do seletor de nível automático e minha solicitação foi simplesmente ignorada. Gostaria de reclamar e solicitar mais uma vez o reparo do seletor de nível automático.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O Purificador não está funcionando! 
+Acionei assistência o mesmo condenou o Purificador! 
+Estou aguardando a substituição! 
+Até o momento não houve nenhum retorno para que seja substituído! </t>
+  </si>
+  <si>
+    <t>O tempo de agendamento para atendimento é muito longo.
+Abri o chamado e só fui atendido 2 semanas depois.
+O elemento filtrante estava muito sujoe e quase não saía mais água do equipamento.
+Muito decepcionado.</t>
+  </si>
+  <si>
+    <t>Demora em substituir o purificador depois da solicitação e, quando substituído, o novo não gelava. No mesmo dia foi solicitado o reparo, faz quase 20 dias que estamos com o equipamento novo sem gelar. O principal motivo de ter um equipamento locado é de ter sua troca o reparo em tempo reduzido. Sem essa vantagem não faz sentido ter este equipamento alugado.</t>
+  </si>
+  <si>
+    <t>Melhorar no cumprimento das realizações das visitas técnicas agendadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Po e muito  difícil  marcar  um horário  para a manutenção,  pelo WhatsApp,  manca consigo  finaliza conversa 
+Fico falando  com um robô, quero falar com uma pessoa,  se for  falar  com um robô,  que seja bem programado por favor. </t>
+  </si>
+  <si>
+    <t>Filtro com problema é simplesmente só podem vir dia 18.
+Resultado: 10 dias sem filtro</t>
+  </si>
+  <si>
+    <t>Motivo (texto-chave detectado)</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>chega sempre no horário de almoço, não faz o combinado + serviço não feito</t>
+  </si>
+  <si>
+    <t>REVISAR</t>
+  </si>
+  <si>
+    <t>demorou 4 dias para atender</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>atendentes despreparados, sem devolutiva de protocolo</t>
+  </si>
+  <si>
+    <t>não terminou o serviço + agenda distante (dia 25)</t>
+  </si>
+  <si>
+    <t>sempre agendam errado por telefone + troca pendente</t>
+  </si>
+  <si>
+    <t>agendaram visita e não cumpriram, remarcaram</t>
+  </si>
+  <si>
+    <t>solicitei diversas vezes, solicitação ignorada</t>
+  </si>
+  <si>
+    <t>aguardando substituição, nenhum retorno</t>
+  </si>
+  <si>
+    <t>atendido 2 semanas depois + quase não saía água</t>
+  </si>
+  <si>
+    <t>equipamento novo sem gelar há 20 dias + demora na troca</t>
+  </si>
+  <si>
+    <t>cumprimento das visitas técnicas agendadas</t>
+  </si>
+  <si>
+    <t>robô no WhatsApp, não consegue finalizar conversa</t>
+  </si>
+  <si>
+    <t>só podem vir dia 18, 10 dias sem filtro</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5059,6 +5175,14 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5118,7 +5242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5143,6 +5267,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5468,7 +5595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1437"/>
+  <dimension ref="A1:M1450"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -5482,10 +5609,12 @@
     <col min="9" max="9" width="28" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.5703125" style="4" customWidth="1"/>
     <col min="11" max="11" width="18.140625" style="4" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="4"/>
+    <col min="12" max="12" width="30" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -5519,8 +5648,14 @@
       <c r="K1" s="4" t="s">
         <v>1438</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="9" t="s">
+        <v>1627</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>1628</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -5555,7 +5690,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -5590,7 +5725,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -5625,7 +5760,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -5660,7 +5795,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -5695,7 +5830,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -5730,7 +5865,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -5765,7 +5900,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -5800,7 +5935,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -5835,7 +5970,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -5870,7 +6005,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -5905,7 +6040,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -5940,7 +6075,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -5975,7 +6110,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -6010,7 +6145,7 @@
         <v>1439</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -55322,7 +55457,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1425" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1425" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1425" s="4">
         <v>429</v>
       </c>
@@ -55357,7 +55492,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1426" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1426" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1426" s="4">
         <v>430</v>
       </c>
@@ -55392,7 +55527,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1427" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1427" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1427" s="4">
         <v>431</v>
       </c>
@@ -55427,7 +55562,7 @@
         <v>1442</v>
       </c>
     </row>
-    <row r="1428" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1428" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1428" s="4">
         <v>432</v>
       </c>
@@ -55462,7 +55597,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1429" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1429" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1429" s="4">
         <v>433</v>
       </c>
@@ -55497,7 +55632,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1430" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1430" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1430" s="4">
         <v>434</v>
       </c>
@@ -55532,7 +55667,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1431" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1431" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1431" s="4">
         <v>435</v>
       </c>
@@ -55567,7 +55702,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="1432" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1432" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1432" s="4">
         <v>436</v>
       </c>
@@ -55602,7 +55737,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1433" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1433" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1433" s="4">
         <v>437</v>
       </c>
@@ -55637,7 +55772,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="1434" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1434" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1434" s="4">
         <v>438</v>
       </c>
@@ -55672,7 +55807,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1435" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1435" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1435" s="4">
         <v>439</v>
       </c>
@@ -55707,7 +55842,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1436" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1436" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1436" s="4">
         <v>440</v>
       </c>
@@ -55742,7 +55877,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1437" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1437" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1437" s="4">
         <v>441</v>
       </c>
@@ -55775,6 +55910,539 @@
       </c>
       <c r="K1437" s="8" t="s">
         <v>1463</v>
+      </c>
+    </row>
+    <row r="1438" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1438" s="4">
+        <v>442</v>
+      </c>
+      <c r="B1438" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1438" s="8">
+        <v>99697</v>
+      </c>
+      <c r="D1438" s="2">
+        <v>46241.620372048608</v>
+      </c>
+      <c r="E1438" s="8" t="s">
+        <v>1610</v>
+      </c>
+      <c r="F1438" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1438" s="8" t="s">
+        <v>1614</v>
+      </c>
+      <c r="H1438" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1438" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1438" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1438" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1438" s="4" t="s">
+        <v>1629</v>
+      </c>
+      <c r="M1438" s="4" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="1439" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1439" s="4">
+        <v>443</v>
+      </c>
+      <c r="B1439" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1439" s="8">
+        <v>113396</v>
+      </c>
+      <c r="D1439" s="2">
+        <v>46241.794543969911</v>
+      </c>
+      <c r="E1439" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1439" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1439" s="8" t="s">
+        <v>1615</v>
+      </c>
+      <c r="H1439" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1439" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1439" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1439" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1439" s="4" t="s">
+        <v>1631</v>
+      </c>
+      <c r="M1439" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1440" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1440" s="4">
+        <v>444</v>
+      </c>
+      <c r="B1440" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1440" s="8">
+        <v>108029</v>
+      </c>
+      <c r="D1440" s="2">
+        <v>46243.6670446875</v>
+      </c>
+      <c r="E1440" s="8" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1440" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1440" s="8" t="s">
+        <v>1616</v>
+      </c>
+      <c r="H1440" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1440" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1440" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1440" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1440" s="4" t="s">
+        <v>1633</v>
+      </c>
+      <c r="M1440" s="4" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="1441" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1441" s="4">
+        <v>445</v>
+      </c>
+      <c r="B1441" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1441" s="8">
+        <v>116676</v>
+      </c>
+      <c r="D1441" s="2">
+        <v>46244.606537280088</v>
+      </c>
+      <c r="E1441" s="8" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1441" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1441" s="8" t="s">
+        <v>1617</v>
+      </c>
+      <c r="H1441" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1441" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1441" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1441" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1441" s="4" t="s">
+        <v>1634</v>
+      </c>
+      <c r="M1441" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1442" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1442" s="4">
+        <v>447</v>
+      </c>
+      <c r="B1442" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1442" s="8">
+        <v>105481</v>
+      </c>
+      <c r="D1442" s="2">
+        <v>46244.637655451392</v>
+      </c>
+      <c r="E1442" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1442" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1442" s="8" t="s">
+        <v>1618</v>
+      </c>
+      <c r="H1442" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1442" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="J1442" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1442" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1442" s="4" t="s">
+        <v>1635</v>
+      </c>
+      <c r="M1442" s="4" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="1443" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1443" s="4">
+        <v>449</v>
+      </c>
+      <c r="B1443" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1443" s="8">
+        <v>114242</v>
+      </c>
+      <c r="D1443" s="2">
+        <v>46244.653732372688</v>
+      </c>
+      <c r="E1443" s="8" t="s">
+        <v>1611</v>
+      </c>
+      <c r="F1443" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1443" s="8" t="s">
+        <v>1619</v>
+      </c>
+      <c r="H1443" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1443" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1443" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1443" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1443" s="4" t="s">
+        <v>1636</v>
+      </c>
+      <c r="M1443" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1444" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1444" s="4">
+        <v>450</v>
+      </c>
+      <c r="B1444" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1444" s="8">
+        <v>114262</v>
+      </c>
+      <c r="D1444" s="2">
+        <v>46244.674947638887</v>
+      </c>
+      <c r="E1444" s="8" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1444" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1444" s="8" t="s">
+        <v>1620</v>
+      </c>
+      <c r="H1444" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1444" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1444" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1444" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1444" s="4" t="s">
+        <v>1637</v>
+      </c>
+      <c r="M1444" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1445" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1445" s="4">
+        <v>452</v>
+      </c>
+      <c r="B1445" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1445" s="8">
+        <v>115579</v>
+      </c>
+      <c r="D1445" s="2">
+        <v>46244.700219062499</v>
+      </c>
+      <c r="E1445" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1445" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1445" s="8" t="s">
+        <v>1621</v>
+      </c>
+      <c r="H1445" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1445" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1445" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1445" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1445" s="4" t="s">
+        <v>1638</v>
+      </c>
+      <c r="M1445" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1446" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1446" s="4">
+        <v>453</v>
+      </c>
+      <c r="B1446" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1446" s="8">
+        <v>108581</v>
+      </c>
+      <c r="D1446" s="2">
+        <v>46244.711498854173</v>
+      </c>
+      <c r="E1446" s="8" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1446" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1446" s="8" t="s">
+        <v>1622</v>
+      </c>
+      <c r="H1446" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1446" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1446" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1446" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1446" s="4" t="s">
+        <v>1639</v>
+      </c>
+      <c r="M1446" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1447" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1447" s="4">
+        <v>454</v>
+      </c>
+      <c r="B1447" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1447" s="8">
+        <v>106871</v>
+      </c>
+      <c r="D1447" s="2">
+        <v>46244.757379641203</v>
+      </c>
+      <c r="E1447" s="8" t="s">
+        <v>1612</v>
+      </c>
+      <c r="F1447" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1447" s="8" t="s">
+        <v>1623</v>
+      </c>
+      <c r="H1447" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1447" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1447" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1447" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1447" s="4" t="s">
+        <v>1640</v>
+      </c>
+      <c r="M1447" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1448" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1448" s="4">
+        <v>455</v>
+      </c>
+      <c r="B1448" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1448" s="8">
+        <v>113979</v>
+      </c>
+      <c r="D1448" s="2">
+        <v>46244.787126689807</v>
+      </c>
+      <c r="E1448" s="8" t="s">
+        <v>1613</v>
+      </c>
+      <c r="F1448" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1448" s="8" t="s">
+        <v>1624</v>
+      </c>
+      <c r="H1448" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1448" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1448" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1448" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1448" s="4" t="s">
+        <v>1641</v>
+      </c>
+      <c r="M1448" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1449" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1449" s="4">
+        <v>456</v>
+      </c>
+      <c r="B1449" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1449" s="8">
+        <v>107921</v>
+      </c>
+      <c r="D1449" s="2">
+        <v>46245.386342928243</v>
+      </c>
+      <c r="E1449" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1449" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1449" s="8" t="s">
+        <v>1625</v>
+      </c>
+      <c r="H1449" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1449" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1449" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1449" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1449" s="4" t="s">
+        <v>1642</v>
+      </c>
+      <c r="M1449" s="4" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1450" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1450" s="4">
+        <v>457</v>
+      </c>
+      <c r="B1450" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1450" s="8">
+        <v>115894</v>
+      </c>
+      <c r="D1450" s="2">
+        <v>46245.535121446759</v>
+      </c>
+      <c r="E1450" s="8" t="s">
+        <v>1576</v>
+      </c>
+      <c r="F1450" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1450" s="8" t="s">
+        <v>1626</v>
+      </c>
+      <c r="H1450" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1450" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1450" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1450" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1450" s="4" t="s">
+        <v>1643</v>
+      </c>
+      <c r="M1450" s="4" t="s">
+        <v>1632</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 12/08/2026  9:20:30,26
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="616" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BEBF561-D19C-459A-89D6-5A7D18CDF1B6}"/>
+  <xr:revisionPtr revIDLastSave="633" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E2BB1C8-DB9A-48AB-9DCD-28A63353E629}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="1920" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1450</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1451</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11630" uniqueCount="1644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11638" uniqueCount="1645">
   <si>
     <t>ID</t>
   </si>
@@ -5154,6 +5154,9 @@
   </si>
   <si>
     <t>só podem vir dia 18, 10 dias sem filtro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boa Tarde ! Colaborar atencioso e educado. Porém, minha insatisfação e com o cilindro de gás, estamos a mais de um ano tentado comprar um cilindro para agua com gás e voces não tem o produto para vender . </t>
   </si>
 </sst>
 </file>
@@ -5595,7 +5598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1450"/>
+  <dimension ref="A1:M1451"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -56445,6 +56448,41 @@
         <v>1632</v>
       </c>
     </row>
+    <row r="1451" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1451" s="4">
+        <v>458</v>
+      </c>
+      <c r="B1451" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1451" s="8">
+        <v>109945</v>
+      </c>
+      <c r="D1451" s="2">
+        <v>46245.77177752315</v>
+      </c>
+      <c r="E1451" s="8" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1451" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1451" s="8" t="s">
+        <v>1644</v>
+      </c>
+      <c r="H1451" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1451" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1451" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1451" s="8" t="s">
+        <v>1441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 17/08/2026 13:30:28,76
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="633" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E2BB1C8-DB9A-48AB-9DCD-28A63353E629}"/>
+  <xr:revisionPtr revIDLastSave="705" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{270A3ED1-7987-4D50-A7AC-16BA09B62C38}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11638" uniqueCount="1645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11738" uniqueCount="1651">
   <si>
     <t>ID</t>
   </si>
@@ -5111,52 +5111,75 @@
     <t>Status</t>
   </si>
   <si>
-    <t>chega sempre no horário de almoço, não faz o combinado + serviço não feito</t>
-  </si>
-  <si>
-    <t>REVISAR</t>
-  </si>
-  <si>
-    <t>demorou 4 dias para atender</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>atendentes despreparados, sem devolutiva de protocolo</t>
-  </si>
-  <si>
-    <t>não terminou o serviço + agenda distante (dia 25)</t>
-  </si>
-  <si>
-    <t>sempre agendam errado por telefone + troca pendente</t>
-  </si>
-  <si>
-    <t>agendaram visita e não cumpriram, remarcaram</t>
-  </si>
-  <si>
-    <t>solicitei diversas vezes, solicitação ignorada</t>
-  </si>
-  <si>
-    <t>aguardando substituição, nenhum retorno</t>
-  </si>
-  <si>
-    <t>atendido 2 semanas depois + quase não saía água</t>
-  </si>
-  <si>
-    <t>equipamento novo sem gelar há 20 dias + demora na troca</t>
-  </si>
-  <si>
-    <t>cumprimento das visitas técnicas agendadas</t>
-  </si>
-  <si>
-    <t>robô no WhatsApp, não consegue finalizar conversa</t>
-  </si>
-  <si>
-    <t>só podem vir dia 18, 10 dias sem filtro</t>
-  </si>
-  <si>
     <t xml:space="preserve">Boa Tarde ! Colaborar atencioso e educado. Porém, minha insatisfação e com o cilindro de gás, estamos a mais de um ano tentado comprar um cilindro para agua com gás e voces não tem o produto para vender . </t>
+  </si>
+  <si>
+    <t>15/08/2026</t>
+  </si>
+  <si>
+    <t>14/08/2026</t>
+  </si>
+  <si>
+    <t>13/08/2026</t>
+  </si>
+  <si>
+    <t>12/08/2026</t>
+  </si>
+  <si>
+    <t>FRQ GOIANIA  GO R01</t>
+  </si>
+  <si>
+    <t>FRQ LIMEIRA SP R04</t>
+  </si>
+  <si>
+    <t>FRQ CAMPINAS R04</t>
+  </si>
+  <si>
+    <t>Falat de compromisso com o horário agendado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não atendem , pedi o atendimento </t>
+  </si>
+  <si>
+    <t>Pq mesmo estando anotado na ordem de serviço, não veio o elemento filtrante NiB gel, o filtro que foi retirado a manutenção tinha sido feita pela metade e um mês depois já precisou de nova manutenção, pois a água estava podre, cheirando muito mal e dentro do aparelho estava cheio de baratas! Espero que esse novo aparelho, esteja sem contaminação , sem baratas ou ovos e que a Culligan verifique aonde são guardados os elementos filtrantes e que haja um cuidado e controle de qualidade melhor!</t>
+  </si>
+  <si>
+    <t>Vieram aqui quarta de manhã dia 12/08 detectaram o furo na mangueira e a prestadora de serviço falou que iriam voltar no mesmo dia a tarde ou até na quinta de manhã, e até agora não vieram resolver o vazamento</t>
+  </si>
+  <si>
+    <t>Porque agendei 2 vezes e não apareceu ninguém. É muita falta de respeito com o tempo do cliente.</t>
+  </si>
+  <si>
+    <t>Na minha opinião, este serviço só compensa  se trocar o filtro a cada 06 meses.
+Fazer uma analise da agua e dizer que esta boa e ficar com um filtro 1ano é tentar economizar</t>
+  </si>
+  <si>
+    <t>De todos os atendimentos de manutenção semestral diria que esse foi o pior e que menos avaliou a real necessidade de troca ou não de peças.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">meu purificador continua com um gosto de metal e continua esquentando muito. nada foi resolvido, só trocaram o filtro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">O prestador de serviço fez o serviço ok, porém deixou sujeira no local, plástico pelo chão, sendo que a lixeira está ao lado do local onde ele fez o serviço. Lamentável. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiquei muito preocupada pela visita, sem crachá de Identificação e sem uniforme.
+A ordem de Serviço não tem nenhuma identificação, sem logomarca, nem endereço ou telefone de contato, não consta o CNPJ da empresa. Após ler toda a Ordem de Serviço, consegui encontrar o nome Culligar, no formato pequeno em uma linha na esquerda da Ordem de Serviço.  Sem telefone para contato. Embora o Técnico tenha sido  muito educado, simpático, respondendo minhas perguntas, não foi o suficiente para me tranquilizar. O que me deixou tranquila foi ele mencionar outros técnicos  da Brastemp conhecido por mim. Friso que o problema não foi o rapaz, mas Ordem de Serviço,  sem dados suficientes, imprecisa, que não passa nenhuma segurança para os clientes.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estou solicitando a quase um mês que me enviem a fatura SEM SENHA, não bate com o meu CPF..
+Até agora não fui atendido.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agendei no período da tarde, chegaram pela manhã no primeiro horario. Deixei subir. 
+Fizeram a manutenção, ok. Mas nao me avisaram que vazou agua embaixo do filtro, ele fica em suporte de madeira em um movél planejado, eleS deixaram cheio de agua embaixo e não avisaram. Só foi notado bem depois, isso estraga o movél. Era algo tão simples era só avisar que molhou, não precisava secar, mas não, fecharam o filtro e colocaram a peça de suporte e não falaram nada. NOTA 0 PARA OS DOIS PROFISSIONAIS QUE ESTIVERAM AQUI. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quase um mês minha purificador  de água não  está gelando,  desde então estou tentando  entrar em contato e não  consigo falar com ser humano,  só robô,  ainda aguardando outro purificador e tb desconto na minha conta que esta muito  caro e tb mal atendido. </t>
+  </si>
+  <si>
+    <t>Porque vocês estão muito desorganizados, enviam o técnico sem fazer uma programação antecipada, sem avisar, e todas as vezes, nesses ultimos meses, tem pego nós desprevenidos, isso demonstra uma total falta de organização e respeito com o cliente!</t>
   </si>
 </sst>
 </file>
@@ -5598,7 +5621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1451"/>
+  <dimension ref="A1:M1465"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -55460,7 +55483,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1425" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1425" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1425" s="4">
         <v>429</v>
       </c>
@@ -55495,7 +55518,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1426" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1426" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1426" s="4">
         <v>430</v>
       </c>
@@ -55530,7 +55553,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1427" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1427" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1427" s="4">
         <v>431</v>
       </c>
@@ -55565,7 +55588,7 @@
         <v>1442</v>
       </c>
     </row>
-    <row r="1428" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1428" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1428" s="4">
         <v>432</v>
       </c>
@@ -55600,7 +55623,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1429" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1429" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1429" s="4">
         <v>433</v>
       </c>
@@ -55635,7 +55658,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1430" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1430" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1430" s="4">
         <v>434</v>
       </c>
@@ -55670,7 +55693,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1431" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1431" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1431" s="4">
         <v>435</v>
       </c>
@@ -55705,7 +55728,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="1432" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1432" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1432" s="4">
         <v>436</v>
       </c>
@@ -55740,7 +55763,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1433" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1433" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1433" s="4">
         <v>437</v>
       </c>
@@ -55775,7 +55798,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="1434" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1434" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1434" s="4">
         <v>438</v>
       </c>
@@ -55810,7 +55833,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1435" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1435" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1435" s="4">
         <v>439</v>
       </c>
@@ -55845,7 +55868,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1436" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1436" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1436" s="4">
         <v>440</v>
       </c>
@@ -55880,7 +55903,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1437" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1437" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1437" s="4">
         <v>441</v>
       </c>
@@ -55915,7 +55938,7 @@
         <v>1463</v>
       </c>
     </row>
-    <row r="1438" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1438" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1438" s="4">
         <v>442</v>
       </c>
@@ -55941,7 +55964,7 @@
         <v>18</v>
       </c>
       <c r="I1438" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="J1438" s="4" t="s">
         <v>1405</v>
@@ -55949,14 +55972,8 @@
       <c r="K1438" s="8" t="s">
         <v>1441</v>
       </c>
-      <c r="L1438" s="4" t="s">
-        <v>1629</v>
-      </c>
-      <c r="M1438" s="4" t="s">
-        <v>1630</v>
-      </c>
-    </row>
-    <row r="1439" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1439" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1439" s="4">
         <v>443</v>
       </c>
@@ -55990,14 +56007,8 @@
       <c r="K1439" s="8" t="s">
         <v>1440</v>
       </c>
-      <c r="L1439" s="4" t="s">
-        <v>1631</v>
-      </c>
-      <c r="M1439" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1440" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1440" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1440" s="4">
         <v>444</v>
       </c>
@@ -56031,14 +56042,8 @@
       <c r="K1440" s="8" t="s">
         <v>1441</v>
       </c>
-      <c r="L1440" s="4" t="s">
-        <v>1633</v>
-      </c>
-      <c r="M1440" s="4" t="s">
-        <v>1630</v>
-      </c>
-    </row>
-    <row r="1441" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1441" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1441" s="4">
         <v>445</v>
       </c>
@@ -56072,14 +56077,8 @@
       <c r="K1441" s="8" t="s">
         <v>1440</v>
       </c>
-      <c r="L1441" s="4" t="s">
-        <v>1634</v>
-      </c>
-      <c r="M1441" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1442" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1442" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1442" s="4">
         <v>447</v>
       </c>
@@ -56113,14 +56112,8 @@
       <c r="K1442" s="8" t="s">
         <v>1441</v>
       </c>
-      <c r="L1442" s="4" t="s">
-        <v>1635</v>
-      </c>
-      <c r="M1442" s="4" t="s">
-        <v>1630</v>
-      </c>
-    </row>
-    <row r="1443" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1443" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1443" s="4">
         <v>449</v>
       </c>
@@ -56154,14 +56147,8 @@
       <c r="K1443" s="8" t="s">
         <v>1440</v>
       </c>
-      <c r="L1443" s="4" t="s">
-        <v>1636</v>
-      </c>
-      <c r="M1443" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1444" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1444" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1444" s="4">
         <v>450</v>
       </c>
@@ -56195,14 +56182,8 @@
       <c r="K1444" s="8" t="s">
         <v>1440</v>
       </c>
-      <c r="L1444" s="4" t="s">
-        <v>1637</v>
-      </c>
-      <c r="M1444" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1445" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1445" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1445" s="4">
         <v>452</v>
       </c>
@@ -56236,14 +56217,8 @@
       <c r="K1445" s="8" t="s">
         <v>1441</v>
       </c>
-      <c r="L1445" s="4" t="s">
-        <v>1638</v>
-      </c>
-      <c r="M1445" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1446" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1446" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1446" s="4">
         <v>453</v>
       </c>
@@ -56277,14 +56252,8 @@
       <c r="K1446" s="8" t="s">
         <v>1440</v>
       </c>
-      <c r="L1446" s="4" t="s">
-        <v>1639</v>
-      </c>
-      <c r="M1446" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1447" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1447" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1447" s="4">
         <v>454</v>
       </c>
@@ -56318,14 +56287,8 @@
       <c r="K1447" s="8" t="s">
         <v>1441</v>
       </c>
-      <c r="L1447" s="4" t="s">
-        <v>1640</v>
-      </c>
-      <c r="M1447" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1448" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1448" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1448" s="4">
         <v>455</v>
       </c>
@@ -56359,14 +56322,8 @@
       <c r="K1448" s="8" t="s">
         <v>1440</v>
       </c>
-      <c r="L1448" s="4" t="s">
-        <v>1641</v>
-      </c>
-      <c r="M1448" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1449" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1449" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1449" s="4">
         <v>456</v>
       </c>
@@ -56400,14 +56357,8 @@
       <c r="K1449" s="8" t="s">
         <v>1440</v>
       </c>
-      <c r="L1449" s="4" t="s">
-        <v>1642</v>
-      </c>
-      <c r="M1449" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1450" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1450" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1450" s="4">
         <v>457</v>
       </c>
@@ -56441,14 +56392,8 @@
       <c r="K1450" s="8" t="s">
         <v>1440</v>
       </c>
-      <c r="L1450" s="4" t="s">
-        <v>1643</v>
-      </c>
-      <c r="M1450" s="4" t="s">
-        <v>1632</v>
-      </c>
-    </row>
-    <row r="1451" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1451" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1451" s="4">
         <v>458</v>
       </c>
@@ -56468,7 +56413,7 @@
         <v>16</v>
       </c>
       <c r="G1451" s="8" t="s">
-        <v>1644</v>
+        <v>1629</v>
       </c>
       <c r="H1451" s="4" t="s">
         <v>13</v>
@@ -56481,6 +56426,496 @@
       </c>
       <c r="K1451" s="8" t="s">
         <v>1441</v>
+      </c>
+    </row>
+    <row r="1452" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1452" s="4">
+        <v>459</v>
+      </c>
+      <c r="B1452" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1452" s="8">
+        <v>121466</v>
+      </c>
+      <c r="D1452" s="8" t="s">
+        <v>1630</v>
+      </c>
+      <c r="E1452" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1452" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1452" s="8" t="s">
+        <v>1637</v>
+      </c>
+      <c r="H1452" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1452" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1452" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1452" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1453" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1453" s="4">
+        <v>460</v>
+      </c>
+      <c r="B1453" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1453" s="8">
+        <v>104421</v>
+      </c>
+      <c r="D1453" s="8" t="s">
+        <v>1630</v>
+      </c>
+      <c r="E1453" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1453" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1453" s="8" t="s">
+        <v>1638</v>
+      </c>
+      <c r="H1453" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1453" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="J1453" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1453" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1454" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1454" s="4">
+        <v>461</v>
+      </c>
+      <c r="B1454" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1454" s="8">
+        <v>122786</v>
+      </c>
+      <c r="D1454" s="8" t="s">
+        <v>1630</v>
+      </c>
+      <c r="E1454" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1454" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1454" s="8" t="s">
+        <v>1639</v>
+      </c>
+      <c r="H1454" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1454" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1454" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1454" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1455" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1455" s="4">
+        <v>462</v>
+      </c>
+      <c r="B1455" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1455" s="8">
+        <v>119382</v>
+      </c>
+      <c r="D1455" s="8" t="s">
+        <v>1630</v>
+      </c>
+      <c r="E1455" s="8" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1455" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1455" s="8" t="s">
+        <v>1640</v>
+      </c>
+      <c r="H1455" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1455" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1455" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1455" s="8" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1456" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1456" s="4">
+        <v>463</v>
+      </c>
+      <c r="B1456" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1456" s="8">
+        <v>119637</v>
+      </c>
+      <c r="D1456" s="8" t="s">
+        <v>1631</v>
+      </c>
+      <c r="E1456" s="8" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F1456" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1456" s="8" t="s">
+        <v>1641</v>
+      </c>
+      <c r="H1456" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1456" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1456" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1456" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1457" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1457" s="4">
+        <v>464</v>
+      </c>
+      <c r="B1457" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1457" s="8">
+        <v>112647</v>
+      </c>
+      <c r="D1457" s="8" t="s">
+        <v>1631</v>
+      </c>
+      <c r="E1457" s="8" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1457" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1457" s="8" t="s">
+        <v>1642</v>
+      </c>
+      <c r="H1457" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1457" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1457" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1457" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1458" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1458" s="4">
+        <v>465</v>
+      </c>
+      <c r="B1458" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1458" s="8">
+        <v>115619</v>
+      </c>
+      <c r="D1458" s="8" t="s">
+        <v>1631</v>
+      </c>
+      <c r="E1458" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1458" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1458" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="H1458" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1458" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1458" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1458" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1459" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1459" s="4">
+        <v>466</v>
+      </c>
+      <c r="B1459" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1459" s="8">
+        <v>113855</v>
+      </c>
+      <c r="D1459" s="8" t="s">
+        <v>1631</v>
+      </c>
+      <c r="E1459" s="8" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1459" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1459" s="8" t="s">
+        <v>1644</v>
+      </c>
+      <c r="H1459" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1459" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1459" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1459" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1460" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1460" s="4">
+        <v>467</v>
+      </c>
+      <c r="B1460" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1460" s="8">
+        <v>112512</v>
+      </c>
+      <c r="D1460" s="8" t="s">
+        <v>1631</v>
+      </c>
+      <c r="E1460" s="8" t="s">
+        <v>803</v>
+      </c>
+      <c r="F1460" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1460" s="8" t="s">
+        <v>1645</v>
+      </c>
+      <c r="H1460" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1460" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1460" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1460" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1461" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1461" s="4">
+        <v>468</v>
+      </c>
+      <c r="B1461" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1461" s="8">
+        <v>97448</v>
+      </c>
+      <c r="D1461" s="8" t="s">
+        <v>1632</v>
+      </c>
+      <c r="E1461" s="8" t="s">
+        <v>1580</v>
+      </c>
+      <c r="F1461" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1461" s="8" t="s">
+        <v>1646</v>
+      </c>
+      <c r="H1461" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1461" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1461" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1461" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1462" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1462" s="4">
+        <v>469</v>
+      </c>
+      <c r="B1462" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1462" s="8">
+        <v>104427</v>
+      </c>
+      <c r="D1462" s="8" t="s">
+        <v>1632</v>
+      </c>
+      <c r="E1462" s="8" t="s">
+        <v>1634</v>
+      </c>
+      <c r="F1462" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1462" s="8" t="s">
+        <v>1647</v>
+      </c>
+      <c r="H1462" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1462" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1462" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1462" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1463" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1463" s="4">
+        <v>470</v>
+      </c>
+      <c r="B1463" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1463" s="8">
+        <v>116197</v>
+      </c>
+      <c r="D1463" s="8" t="s">
+        <v>1632</v>
+      </c>
+      <c r="E1463" s="8" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1463" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1463" s="8" t="s">
+        <v>1648</v>
+      </c>
+      <c r="H1463" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1463" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1463" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1463" s="8" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1464" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1464" s="4">
+        <v>471</v>
+      </c>
+      <c r="B1464" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1464" s="8">
+        <v>117844</v>
+      </c>
+      <c r="D1464" s="8" t="s">
+        <v>1633</v>
+      </c>
+      <c r="E1464" s="8" t="s">
+        <v>1635</v>
+      </c>
+      <c r="F1464" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1464" s="8" t="s">
+        <v>1649</v>
+      </c>
+      <c r="H1464" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1464" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1464" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1464" s="8" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1465" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1465" s="4">
+        <v>472</v>
+      </c>
+      <c r="B1465" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1465" s="8">
+        <v>104357</v>
+      </c>
+      <c r="D1465" s="8" t="s">
+        <v>1633</v>
+      </c>
+      <c r="E1465" s="8" t="s">
+        <v>1636</v>
+      </c>
+      <c r="F1465" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1465" s="8" t="s">
+        <v>1650</v>
+      </c>
+      <c r="H1465" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1465" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1465" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1465" s="8" t="s">
+        <v>1442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 24/08/2026  9:48:25,95
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="705" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{270A3ED1-7987-4D50-A7AC-16BA09B62C38}"/>
+  <xr:revisionPtr revIDLastSave="907" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD3975A2-3AB1-4DF1-A5DB-71AE92081015}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23880" yWindow="1920" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11738" uniqueCount="1651">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12218" uniqueCount="1741">
   <si>
     <t>ID</t>
   </si>
@@ -5180,6 +5180,288 @@
   </si>
   <si>
     <t>Porque vocês estão muito desorganizados, enviam o técnico sem fazer uma programação antecipada, sem avisar, e todas as vezes, nesses ultimos meses, tem pego nós desprevenidos, isso demonstra uma total falta de organização e respeito com o cliente!</t>
+  </si>
+  <si>
+    <t>FRQ MOGI GUACU SP R02</t>
+  </si>
+  <si>
+    <t>FRQ BRAGANCA PAULISTA SP R06</t>
+  </si>
+  <si>
+    <t>FRQ FLORIPA SC R01 - MATRIZ</t>
+  </si>
+  <si>
+    <t>FRQ CAMPINAS R03</t>
+  </si>
+  <si>
+    <t>FRQ CURITIBA PR R06</t>
+  </si>
+  <si>
+    <t>Manutenção Preventiva</t>
+  </si>
+  <si>
+    <t>Troca</t>
+  </si>
+  <si>
+    <t>Somos clientes antigos.
+Após a troca do filtro na semana passada (13/8), água esta com um gosto horrível!
+De química!
+Sempre prezamos pelo sabor da nossa água, mas desta vez!
+Que arrependimento em realizar a manutenção.
+Pra consertar agenda é super complicada.
+Questionamos até se este filtro novo mesmo!</t>
+  </si>
+  <si>
+    <t>Dei essa classificação por conta da resolução da questão da troca do bebedouro, muito tempo pra esperar a solução do problema, quanto ao técnico dou 10, abriu o bebedouro, limpou, explicou e até mesmo disse que falaria com supervisor para adiantar a troca, por meu marido já cancelaria pq 30 dias pra resolver é muito tempo .</t>
+  </si>
+  <si>
+    <t>confusão nos pagamentos da transição, duas visitas não realizadas (10h de espera em vão)</t>
+  </si>
+  <si>
+    <t>Boa tarde,
+Embora o atendimento da equipe de manutenção tenha sido satisfatório, o problema persiste, pois os reparos realizados não estão solucionando a falha de forma satisfatória  .Já solicitei anteriormente a substituição do aparelho, que apresenta desgaste decorrente do tempo de uso e do funcionamento contínuo, mas até o momento não fui atendido.
+Continuo aguardando obg</t>
+  </si>
+  <si>
+    <t>Pela segunda vez recebo a visita técnica para reparo e os técnicos não resolveram os problemas,  mesmo eu informando na chamada o tipo de problema. Estou sem utilizar o filtro a mais de 15 dias. Ficaram de ir trocar o filtro. No ano passado foi igual o mesmo problema!</t>
+  </si>
+  <si>
+    <t>O serviço foi agendado para a sexta feira última, não apareceu ninguém no fia combinado, além disso vocês  me informaram que a visita tinha sido feita.</t>
+  </si>
+  <si>
+    <t>Aparelho não sai agua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A conta não chega ,atrasa tudo,quero cancelar </t>
+  </si>
+  <si>
+    <t>O técnico veio fora do horario previsto.</t>
+  </si>
+  <si>
+    <t>Péssimo. O técnico foi 2x na minha casa e a minha água continua quente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falta de item para fazer manutenção exemplo: FILTRO
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boa tarde. Eu ja fui cliente por 7 anos no RJ e tinha esse mesmo modelo em casa, o filtro foi instalado ontem e hj qdo comecei a usar verifiquei que na retirada da água, esta fazendo um barulho horrível na hora que aperta o botão para parar a água. Nao sei se é defeito, mas muito estranho. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">O equipamento está fazendo um barrulho diferente em funcionamento, e a pessoa que foi dar a manutenção não fez nada, disse que é normal. Achei muito grosseiro da parte dele, e também está claro, que o equipamento não está normal e que vai dar mais problemas se não for resolvido. 
+Detalhe: eu tenho o contrato do equipamento para meus avós, então, talvez ele teve o descaso por ser idosos. </t>
+  </si>
+  <si>
+    <t>Eu solicitei a manutenção semestral porque não houve da parte de vocês manifestação para esse serviço. Aproveitei e informei que meu purificador estava com o fluxo de água comprometido e que a água não estava saindo gelada somente fresca. O tecnico foi fazer o serviço e a agua continua tépida e o fluxo melhorou mas não voltou ao normal. Solicitei nova visita e remarcaram para o dia 26 de agosto!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serviço péssimo. A máquina está com problema sem funcionar desde o dia que foi instalada e não resolvem. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fizemos agendamento com um mês de antecedência e não compareceram, tivemos que remarcar a visita do técnico não durou 5 minutos. Não passou nenhum retorno sobre a visita, nem nada. Sistema falho para tentar avisar que não veio ninguém na visita, falava repetidamente da visita que já havia passado a data. </t>
+  </si>
+  <si>
+    <t>Péssimo atendimento. Foi marcado para o dia 12/08 vieram no dia 11/08 sem aviso prévio. 
+ Funcionário irritado, pois foi perguntado pque da mudança respondeu: se a Sra. quiser eu não faço nada e volto amanhã se der. ?????</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tecnico foi em casa, nao resolveu o problema, deixou o filtro vazando dizendo que voltaria na segunda feira e nunca mais voltou.
+Meu filtro agora continua sem agua gelada e passou a alagar minha cozinha </t>
+  </si>
+  <si>
+    <t>o técnico não compareceu para realizar o serviço.</t>
+  </si>
+  <si>
+    <t>Mais uma vez o problema não foi resolvido. E não tive resposta inclusive sobre o móvel danificado.</t>
+  </si>
+  <si>
+    <t>Não gostei do serviço prestado. O técnico não encaixou a frente do meu purificador corretamente! E assim a bandeja de suporte para copos e garrafas também fica mal encaixada. Um absurdo! Pois penso que o técnico não deveria terminar o serviço e ir embora antes de verificar se tudo estava perfeitamente encaixado! Fiquei muito insatisfeita!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não foi deixado nenhum documento ou relatório do que foi feito. O recibo apenas pediu a Recepcionista para sssinar e não deixou nada </t>
+  </si>
+  <si>
+    <t xml:space="preserve">O técnico nunca vem no dia marcado e termina atrapalhando a rotina ou a manutenção não ocorre </t>
+  </si>
+  <si>
+    <t>Não aconteceu. Fiquei esperando o técnico que não apareceu, não deu satisfação. No dia seguinte entrei em contato e simplesmente fui informado que nada poderia ser feito, pois a empresa de assistência é "terceirizada". Pergunto: o que eu tenho a ver com a forma de trabalho de vocês? Lamentável. Estou até agora esperando algum contato.</t>
+  </si>
+  <si>
+    <t>Os motivos foram declarados na central de atendimento.</t>
+  </si>
+  <si>
+    <t>FALTA DE TRANSPARENCIA COM O CLIENTE</t>
+  </si>
+  <si>
+    <t>PORQUE AGENDAMOS PARA A PARTE DA TARDE E O TÉCNICO VEIO AS 10 HS DA MANHÃ….</t>
+  </si>
+  <si>
+    <t>Péssimo agendamento. Não cumprem prazo. Os profissionais não têm hora pra chegar, independentemente de ter havido, previamente, um agendamento, fora a expectativa de não comparecerem no dia marcado, como aconteceu, recentemente, comigo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muito ruim , estava agendado entre 8:00 e 13:00 chegou 15:00 além disso produto já parou de funcionar </t>
+  </si>
+  <si>
+    <t>O purificador com vazamento por baixo o técnico já veio duas vezes e não resolveu. Tem danos no móvel.</t>
+  </si>
+  <si>
+    <t>bom dia entalação errada, comuniquei ate agora não resolveu&amp;gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Já alugo o aparelho há muito anos,mas tive problemas na última visita técnica agendada. O técnico não tinha a senha que foi enviada. Achei muita deorganização.</t>
+  </si>
+  <si>
+    <t>Não gostei do atendimento  que não durou nem 5 minutos, a manutenção já foi melhor, hj só cola selo</t>
+  </si>
+  <si>
+    <t>enviam técnico sem avisar, pegam desprevenido</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>conta muito caro + não gela + só robô</t>
+  </si>
+  <si>
+    <t>REVISAR</t>
+  </si>
+  <si>
+    <t>deixaram água embaixo e não avisaram</t>
+  </si>
+  <si>
+    <t>pede fatura sem senha, não é atendido</t>
+  </si>
+  <si>
+    <t>sem crachá e sem uniforme</t>
+  </si>
+  <si>
+    <t>deixou sujeira e plástico no chão</t>
+  </si>
+  <si>
+    <t>gosto de metal + esquentando muito</t>
+  </si>
+  <si>
+    <t>não avaliou necessidade de troca de peças</t>
+  </si>
+  <si>
+    <t>não trocou filtro, ficou 1 ano</t>
+  </si>
+  <si>
+    <t>agendei 2 vezes e não apareceu ninguém</t>
+  </si>
+  <si>
+    <t>disseram que voltariam e não vieram</t>
+  </si>
+  <si>
+    <t>não veio o elemento filtrante + água podre</t>
+  </si>
+  <si>
+    <t>não atendem, pedi o atendimento</t>
+  </si>
+  <si>
+    <t>falta de compromisso com horário agendado</t>
+  </si>
+  <si>
+    <t>água com gosto de química após troca</t>
+  </si>
+  <si>
+    <t>30 dias esperando troca do bebedouro</t>
+  </si>
+  <si>
+    <t>duas visitas não realizadas, 10h de espera</t>
+  </si>
+  <si>
+    <t>reparos não solucionam, troca não atendida</t>
+  </si>
+  <si>
+    <t>segunda vez sem resolver, mesmo problema</t>
+  </si>
+  <si>
+    <t>ninguém apareceu e informaram visita feita</t>
+  </si>
+  <si>
+    <t>aparelho não sai água</t>
+  </si>
+  <si>
+    <t>conta não chega, quer cancelar</t>
+  </si>
+  <si>
+    <t>técnico veio fora do horário previsto</t>
+  </si>
+  <si>
+    <t>água continua quente após 2 visitas</t>
+  </si>
+  <si>
+    <t>falta de item para manutenção: filtro</t>
+  </si>
+  <si>
+    <t>barulho horrível ao apertar o botão</t>
+  </si>
+  <si>
+    <t>não fez nada pelo ruído + achei grosseiro</t>
+  </si>
+  <si>
+    <t>água continua tépida + fluxo comprometido</t>
+  </si>
+  <si>
+    <t>sem funcionar desde a instalação</t>
+  </si>
+  <si>
+    <t>preço alto</t>
+  </si>
+  <si>
+    <t>não compareceram + visita de 5 minutos</t>
+  </si>
+  <si>
+    <t>vieram um dia antes sem aviso + irritado</t>
+  </si>
+  <si>
+    <t>deixou o filtro vazando, alagou cozinha</t>
+  </si>
+  <si>
+    <t>técnico não compareceu</t>
+  </si>
+  <si>
+    <t>mais uma vez o problema não foi resolvido</t>
+  </si>
+  <si>
+    <t>não encaixou a frente do purificador</t>
+  </si>
+  <si>
+    <t>não deixou relatório nem comprovante</t>
+  </si>
+  <si>
+    <t>nunca vem no dia marcado</t>
+  </si>
+  <si>
+    <t>não aconteceu, técnico não apareceu</t>
+  </si>
+  <si>
+    <t>motivos declarados na central</t>
+  </si>
+  <si>
+    <t>falta de transparência com o cliente</t>
+  </si>
+  <si>
+    <t>agendado à tarde, veio 10h da manhã</t>
+  </si>
+  <si>
+    <t>não comparecem no dia marcado</t>
+  </si>
+  <si>
+    <t>agendado 8-13h chegou 15h + parou de funcionar</t>
+  </si>
+  <si>
+    <t>vazamento por baixo, 2 visitas sem resolver</t>
+  </si>
+  <si>
+    <t>instalação errada, comuniquei e não resolveu</t>
+  </si>
+  <si>
+    <t>técnico não tinha a senha enviada</t>
+  </si>
+  <si>
+    <t>atendimento não durou 5 minutos, só cola selo</t>
   </si>
 </sst>
 </file>
@@ -5268,7 +5550,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5296,6 +5578,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5621,7 +5906,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1465"/>
+  <dimension ref="A1:M1513"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -56603,7 +56888,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1457" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1457" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1457" s="4">
         <v>464</v>
       </c>
@@ -56638,7 +56923,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1458" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1458" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1458" s="4">
         <v>465</v>
       </c>
@@ -56673,7 +56958,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1459" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1459" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1459" s="4">
         <v>466</v>
       </c>
@@ -56708,7 +56993,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1460" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1460" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1460" s="4">
         <v>467</v>
       </c>
@@ -56743,7 +57028,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1461" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1461" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1461" s="4">
         <v>468</v>
       </c>
@@ -56778,7 +57063,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1462" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1462" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1462" s="4">
         <v>469</v>
       </c>
@@ -56813,7 +57098,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1463" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1463" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1463" s="4">
         <v>470</v>
       </c>
@@ -56848,7 +57133,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="1464" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1464" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1464" s="4">
         <v>471</v>
       </c>
@@ -56883,7 +57168,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="1465" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1465" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1465" s="4">
         <v>472</v>
       </c>
@@ -56916,6 +57201,1974 @@
       </c>
       <c r="K1465" s="8" t="s">
         <v>1442</v>
+      </c>
+    </row>
+    <row r="1466" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1466" s="4">
+        <v>473</v>
+      </c>
+      <c r="B1466" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1466" s="8">
+        <v>104357</v>
+      </c>
+      <c r="D1466" s="10">
+        <v>46246.477436666668</v>
+      </c>
+      <c r="E1466" s="8" t="s">
+        <v>1636</v>
+      </c>
+      <c r="F1466" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1466" s="8" t="s">
+        <v>1650</v>
+      </c>
+      <c r="H1466" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1466" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1466" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1466" s="8" t="s">
+        <v>1442</v>
+      </c>
+      <c r="L1466" s="4" t="s">
+        <v>1691</v>
+      </c>
+      <c r="M1466" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1467" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1467" s="4">
+        <v>474</v>
+      </c>
+      <c r="B1467" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1467" s="8">
+        <v>117844</v>
+      </c>
+      <c r="D1467" s="10">
+        <v>46246.860933148149</v>
+      </c>
+      <c r="E1467" s="8" t="s">
+        <v>1635</v>
+      </c>
+      <c r="F1467" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1467" s="8" t="s">
+        <v>1649</v>
+      </c>
+      <c r="H1467" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1467" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1467" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1467" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1467" s="4" t="s">
+        <v>1693</v>
+      </c>
+      <c r="M1467" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1468" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1468" s="4">
+        <v>475</v>
+      </c>
+      <c r="B1468" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1468" s="8">
+        <v>116197</v>
+      </c>
+      <c r="D1468" s="10">
+        <v>46247.73844645833</v>
+      </c>
+      <c r="E1468" s="8" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1468" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1468" s="8" t="s">
+        <v>1648</v>
+      </c>
+      <c r="H1468" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1468" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1468" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1468" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1468" s="4" t="s">
+        <v>1695</v>
+      </c>
+      <c r="M1468" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1469" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1469" s="4">
+        <v>476</v>
+      </c>
+      <c r="B1469" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1469" s="8">
+        <v>104427</v>
+      </c>
+      <c r="D1469" s="10">
+        <v>46247.761227499999</v>
+      </c>
+      <c r="E1469" s="8" t="s">
+        <v>1634</v>
+      </c>
+      <c r="F1469" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1469" s="8" t="s">
+        <v>1647</v>
+      </c>
+      <c r="H1469" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1469" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1469" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1469" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1469" s="4" t="s">
+        <v>1696</v>
+      </c>
+      <c r="M1469" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1470" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1470" s="4">
+        <v>477</v>
+      </c>
+      <c r="B1470" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1470" s="8">
+        <v>97448</v>
+      </c>
+      <c r="D1470" s="10">
+        <v>46247.76924115741</v>
+      </c>
+      <c r="E1470" s="8" t="s">
+        <v>1580</v>
+      </c>
+      <c r="F1470" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1470" s="8" t="s">
+        <v>1646</v>
+      </c>
+      <c r="H1470" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1470" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1470" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1470" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1470" s="4" t="s">
+        <v>1697</v>
+      </c>
+      <c r="M1470" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1471" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1471" s="4">
+        <v>478</v>
+      </c>
+      <c r="B1471" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1471" s="8">
+        <v>112512</v>
+      </c>
+      <c r="D1471" s="10">
+        <v>46248.768450856478</v>
+      </c>
+      <c r="E1471" s="8" t="s">
+        <v>803</v>
+      </c>
+      <c r="F1471" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1471" s="8" t="s">
+        <v>1645</v>
+      </c>
+      <c r="H1471" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1471" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1471" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1471" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1471" s="4" t="s">
+        <v>1698</v>
+      </c>
+      <c r="M1471" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1472" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1472" s="4">
+        <v>479</v>
+      </c>
+      <c r="B1472" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1472" s="8">
+        <v>113855</v>
+      </c>
+      <c r="D1472" s="10">
+        <v>46248.78429275463</v>
+      </c>
+      <c r="E1472" s="8" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1472" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1472" s="8" t="s">
+        <v>1644</v>
+      </c>
+      <c r="H1472" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1472" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1472" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1472" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1472" s="4" t="s">
+        <v>1699</v>
+      </c>
+      <c r="M1472" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1473" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1473" s="4">
+        <v>480</v>
+      </c>
+      <c r="B1473" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1473" s="8">
+        <v>115619</v>
+      </c>
+      <c r="D1473" s="10">
+        <v>46248.846609004628</v>
+      </c>
+      <c r="E1473" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1473" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1473" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="H1473" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1473" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1473" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1473" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1473" s="4" t="s">
+        <v>1700</v>
+      </c>
+      <c r="M1473" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1474" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1474" s="4">
+        <v>481</v>
+      </c>
+      <c r="B1474" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1474" s="8">
+        <v>112647</v>
+      </c>
+      <c r="D1474" s="10">
+        <v>46248.886021979168</v>
+      </c>
+      <c r="E1474" s="8" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1474" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1474" s="8" t="s">
+        <v>1642</v>
+      </c>
+      <c r="H1474" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1474" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1474" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1474" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1474" s="4" t="s">
+        <v>1701</v>
+      </c>
+      <c r="M1474" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1475" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1475" s="4">
+        <v>482</v>
+      </c>
+      <c r="B1475" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1475" s="8">
+        <v>119637</v>
+      </c>
+      <c r="D1475" s="10">
+        <v>46248.921772291673</v>
+      </c>
+      <c r="E1475" s="8" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F1475" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1475" s="8" t="s">
+        <v>1641</v>
+      </c>
+      <c r="H1475" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1475" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1475" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1475" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1475" s="4" t="s">
+        <v>1702</v>
+      </c>
+      <c r="M1475" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1476" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1476" s="4">
+        <v>483</v>
+      </c>
+      <c r="B1476" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1476" s="8">
+        <v>119382</v>
+      </c>
+      <c r="D1476" s="10">
+        <v>46249.484861122677</v>
+      </c>
+      <c r="E1476" s="8" t="s">
+        <v>1246</v>
+      </c>
+      <c r="F1476" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1476" s="8" t="s">
+        <v>1640</v>
+      </c>
+      <c r="H1476" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1476" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1476" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1476" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1476" s="4" t="s">
+        <v>1703</v>
+      </c>
+      <c r="M1476" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1477" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1477" s="4">
+        <v>484</v>
+      </c>
+      <c r="B1477" s="8" t="s">
+        <v>1657</v>
+      </c>
+      <c r="C1477" s="8">
+        <v>122786</v>
+      </c>
+      <c r="D1477" s="10">
+        <v>46249.539972361112</v>
+      </c>
+      <c r="E1477" s="8" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1477" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1477" s="8" t="s">
+        <v>1639</v>
+      </c>
+      <c r="H1477" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1477" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1477" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1477" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1477" s="4" t="s">
+        <v>1704</v>
+      </c>
+      <c r="M1477" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1478" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1478" s="4">
+        <v>485</v>
+      </c>
+      <c r="B1478" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1478" s="8">
+        <v>104421</v>
+      </c>
+      <c r="D1478" s="10">
+        <v>46249.68085780093</v>
+      </c>
+      <c r="E1478" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1478" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1478" s="8" t="s">
+        <v>1638</v>
+      </c>
+      <c r="H1478" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1478" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="J1478" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1478" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1478" s="4" t="s">
+        <v>1705</v>
+      </c>
+      <c r="M1478" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1479" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1479" s="4">
+        <v>486</v>
+      </c>
+      <c r="B1479" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1479" s="8">
+        <v>121466</v>
+      </c>
+      <c r="D1479" s="10">
+        <v>46249.716209664351</v>
+      </c>
+      <c r="E1479" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1479" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1479" s="8" t="s">
+        <v>1637</v>
+      </c>
+      <c r="H1479" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1479" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1479" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1479" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1479" s="4" t="s">
+        <v>1706</v>
+      </c>
+      <c r="M1479" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1480" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1480" s="4">
+        <v>487</v>
+      </c>
+      <c r="B1480" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1480" s="8">
+        <v>121020</v>
+      </c>
+      <c r="D1480" s="10">
+        <v>46251.548014814813</v>
+      </c>
+      <c r="E1480" s="8" t="s">
+        <v>1651</v>
+      </c>
+      <c r="F1480" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1480" s="8" t="s">
+        <v>1658</v>
+      </c>
+      <c r="H1480" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1480" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1480" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1480" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1480" s="4" t="s">
+        <v>1707</v>
+      </c>
+      <c r="M1480" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1481" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1481" s="4">
+        <v>488</v>
+      </c>
+      <c r="B1481" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1481" s="8">
+        <v>110872</v>
+      </c>
+      <c r="D1481" s="10">
+        <v>46251.59071384259</v>
+      </c>
+      <c r="E1481" s="8" t="s">
+        <v>1610</v>
+      </c>
+      <c r="F1481" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1481" s="8" t="s">
+        <v>1659</v>
+      </c>
+      <c r="H1481" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1481" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1481" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1481" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1481" s="4" t="s">
+        <v>1708</v>
+      </c>
+      <c r="M1481" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1482" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1482" s="4">
+        <v>489</v>
+      </c>
+      <c r="B1482" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1482" s="8">
+        <v>119549</v>
+      </c>
+      <c r="D1482" s="10">
+        <v>46251.595791782413</v>
+      </c>
+      <c r="E1482" s="8" t="s">
+        <v>1447</v>
+      </c>
+      <c r="F1482" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1482" s="8" t="s">
+        <v>1660</v>
+      </c>
+      <c r="H1482" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1482" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1482" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1482" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1482" s="4" t="s">
+        <v>1709</v>
+      </c>
+      <c r="M1482" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1483" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1483" s="4">
+        <v>490</v>
+      </c>
+      <c r="B1483" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1483" s="8">
+        <v>114435</v>
+      </c>
+      <c r="D1483" s="10">
+        <v>46251.644513576393</v>
+      </c>
+      <c r="E1483" s="8" t="s">
+        <v>1652</v>
+      </c>
+      <c r="F1483" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1483" s="8" t="s">
+        <v>1661</v>
+      </c>
+      <c r="H1483" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1483" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1483" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1483" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1483" s="4" t="s">
+        <v>1710</v>
+      </c>
+      <c r="M1483" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1484" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1484" s="4">
+        <v>491</v>
+      </c>
+      <c r="B1484" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1484" s="8">
+        <v>116426</v>
+      </c>
+      <c r="D1484" s="10">
+        <v>46251.657401446762</v>
+      </c>
+      <c r="E1484" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1484" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1484" s="8" t="s">
+        <v>1662</v>
+      </c>
+      <c r="H1484" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1484" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1484" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1484" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1484" s="4" t="s">
+        <v>1711</v>
+      </c>
+      <c r="M1484" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1485" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1485" s="4">
+        <v>492</v>
+      </c>
+      <c r="B1485" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1485" s="8">
+        <v>96354</v>
+      </c>
+      <c r="D1485" s="10">
+        <v>46251.660639374997</v>
+      </c>
+      <c r="E1485" s="8" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1485" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1485" s="8" t="s">
+        <v>1663</v>
+      </c>
+      <c r="H1485" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1485" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1485" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1485" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1485" s="4" t="s">
+        <v>1712</v>
+      </c>
+      <c r="M1485" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1486" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1486" s="4">
+        <v>493</v>
+      </c>
+      <c r="B1486" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1486" s="8">
+        <v>116408</v>
+      </c>
+      <c r="D1486" s="10">
+        <v>46251.675366412041</v>
+      </c>
+      <c r="E1486" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1486" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1486" s="8" t="s">
+        <v>1664</v>
+      </c>
+      <c r="H1486" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1486" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="J1486" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1486" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1486" s="4" t="s">
+        <v>1713</v>
+      </c>
+      <c r="M1486" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1487" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1487" s="4">
+        <v>494</v>
+      </c>
+      <c r="B1487" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1487" s="8">
+        <v>123194</v>
+      </c>
+      <c r="D1487" s="10">
+        <v>46251.698660752307</v>
+      </c>
+      <c r="E1487" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1487" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1487" s="8" t="s">
+        <v>1665</v>
+      </c>
+      <c r="H1487" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1487" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1487" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1487" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1487" s="4" t="s">
+        <v>1714</v>
+      </c>
+      <c r="M1487" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1488" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1488" s="4">
+        <v>495</v>
+      </c>
+      <c r="B1488" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1488" s="8">
+        <v>110065</v>
+      </c>
+      <c r="D1488" s="10">
+        <v>46251.738354201392</v>
+      </c>
+      <c r="E1488" s="8" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1488" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1488" s="8" t="s">
+        <v>1666</v>
+      </c>
+      <c r="H1488" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1488" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1488" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1488" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1488" s="4" t="s">
+        <v>1715</v>
+      </c>
+      <c r="M1488" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1489" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1489" s="4">
+        <v>496</v>
+      </c>
+      <c r="B1489" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1489" s="8">
+        <v>119204</v>
+      </c>
+      <c r="D1489" s="10">
+        <v>46251.839549166667</v>
+      </c>
+      <c r="E1489" s="8" t="s">
+        <v>1613</v>
+      </c>
+      <c r="F1489" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1489" s="8" t="s">
+        <v>1667</v>
+      </c>
+      <c r="H1489" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1489" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1489" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1489" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1489" s="4" t="s">
+        <v>1716</v>
+      </c>
+      <c r="M1489" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1490" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1490" s="4">
+        <v>497</v>
+      </c>
+      <c r="B1490" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1490" s="8">
+        <v>116632</v>
+      </c>
+      <c r="D1490" s="10">
+        <v>46252.58895109954</v>
+      </c>
+      <c r="E1490" s="8" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1490" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1490" s="8" t="s">
+        <v>1668</v>
+      </c>
+      <c r="H1490" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1490" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1490" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1490" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1490" s="4" t="s">
+        <v>1717</v>
+      </c>
+      <c r="M1490" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1491" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1491" s="4">
+        <v>498</v>
+      </c>
+      <c r="B1491" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1491" s="8">
+        <v>122445</v>
+      </c>
+      <c r="D1491" s="10">
+        <v>46252.756570995371</v>
+      </c>
+      <c r="E1491" s="8" t="s">
+        <v>1653</v>
+      </c>
+      <c r="F1491" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1491" s="8" t="s">
+        <v>1669</v>
+      </c>
+      <c r="H1491" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1491" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1491" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1491" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1491" s="4" t="s">
+        <v>1718</v>
+      </c>
+      <c r="M1491" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1492" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1492" s="4">
+        <v>499</v>
+      </c>
+      <c r="B1492" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1492" s="8">
+        <v>121871</v>
+      </c>
+      <c r="D1492" s="10">
+        <v>46252.826207824073</v>
+      </c>
+      <c r="E1492" s="8" t="s">
+        <v>1654</v>
+      </c>
+      <c r="F1492" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1492" s="8" t="s">
+        <v>1670</v>
+      </c>
+      <c r="H1492" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1492" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1492" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1492" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1492" s="4" t="s">
+        <v>1719</v>
+      </c>
+      <c r="M1492" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1493" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1493" s="4">
+        <v>500</v>
+      </c>
+      <c r="B1493" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1493" s="8">
+        <v>119520</v>
+      </c>
+      <c r="D1493" s="10">
+        <v>46252.867391435182</v>
+      </c>
+      <c r="E1493" s="8" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F1493" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1493" s="8" t="s">
+        <v>1671</v>
+      </c>
+      <c r="H1493" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1493" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1493" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1493" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1493" s="4" t="s">
+        <v>1720</v>
+      </c>
+      <c r="M1493" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1494" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1494" s="4">
+        <v>501</v>
+      </c>
+      <c r="B1494" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1494" s="8">
+        <v>120161</v>
+      </c>
+      <c r="D1494" s="10">
+        <v>46252.950519965278</v>
+      </c>
+      <c r="E1494" s="8" t="s">
+        <v>1580</v>
+      </c>
+      <c r="F1494" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1494" s="8" t="s">
+        <v>1672</v>
+      </c>
+      <c r="H1494" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1494" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1494" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1494" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1494" s="4" t="s">
+        <v>1721</v>
+      </c>
+      <c r="M1494" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1495" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1495" s="4">
+        <v>502</v>
+      </c>
+      <c r="B1495" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1495" s="8">
+        <v>118051</v>
+      </c>
+      <c r="D1495" s="10">
+        <v>46253.711167974543</v>
+      </c>
+      <c r="E1495" s="8" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1495" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1495" s="8" t="s">
+        <v>1189</v>
+      </c>
+      <c r="H1495" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1495" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1495" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1495" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1495" s="4" t="s">
+        <v>1722</v>
+      </c>
+      <c r="M1495" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1496" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1496" s="4">
+        <v>503</v>
+      </c>
+      <c r="B1496" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1496" s="8">
+        <v>118660</v>
+      </c>
+      <c r="D1496" s="10">
+        <v>46253.793205069444</v>
+      </c>
+      <c r="E1496" s="8" t="s">
+        <v>1447</v>
+      </c>
+      <c r="F1496" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1496" s="8" t="s">
+        <v>1673</v>
+      </c>
+      <c r="H1496" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1496" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1496" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1496" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1496" s="4" t="s">
+        <v>1723</v>
+      </c>
+      <c r="M1496" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1497" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1497" s="4">
+        <v>504</v>
+      </c>
+      <c r="B1497" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1497" s="8">
+        <v>119228</v>
+      </c>
+      <c r="D1497" s="10">
+        <v>46253.828614652783</v>
+      </c>
+      <c r="E1497" s="8" t="s">
+        <v>1655</v>
+      </c>
+      <c r="F1497" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1497" s="8" t="s">
+        <v>1674</v>
+      </c>
+      <c r="H1497" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1497" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1497" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1497" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1497" s="4" t="s">
+        <v>1724</v>
+      </c>
+      <c r="M1497" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1498" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1498" s="4">
+        <v>505</v>
+      </c>
+      <c r="B1498" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1498" s="8">
+        <v>118868</v>
+      </c>
+      <c r="D1498" s="10">
+        <v>46254.568633726849</v>
+      </c>
+      <c r="E1498" s="8" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1498" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1498" s="8" t="s">
+        <v>1675</v>
+      </c>
+      <c r="H1498" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1498" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1498" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1498" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1498" s="4" t="s">
+        <v>1725</v>
+      </c>
+      <c r="M1498" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1499" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1499" s="4">
+        <v>506</v>
+      </c>
+      <c r="B1499" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1499" s="8">
+        <v>112487</v>
+      </c>
+      <c r="D1499" s="10">
+        <v>46254.612892476849</v>
+      </c>
+      <c r="E1499" s="8" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1499" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1499" s="8" t="s">
+        <v>1676</v>
+      </c>
+      <c r="H1499" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1499" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1499" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1499" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1499" s="4" t="s">
+        <v>1726</v>
+      </c>
+      <c r="M1499" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1500" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1500" s="4">
+        <v>507</v>
+      </c>
+      <c r="B1500" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1500" s="8">
+        <v>120111</v>
+      </c>
+      <c r="D1500" s="10">
+        <v>46254.670405370372</v>
+      </c>
+      <c r="E1500" s="8" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1500" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1500" s="8" t="s">
+        <v>1677</v>
+      </c>
+      <c r="H1500" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1500" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1500" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1500" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1500" s="4" t="s">
+        <v>1727</v>
+      </c>
+      <c r="M1500" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1501" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1501" s="4">
+        <v>508</v>
+      </c>
+      <c r="B1501" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1501" s="8">
+        <v>109186</v>
+      </c>
+      <c r="D1501" s="10">
+        <v>46254.880398946763</v>
+      </c>
+      <c r="E1501" s="8" t="s">
+        <v>1256</v>
+      </c>
+      <c r="F1501" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1501" s="8" t="s">
+        <v>1678</v>
+      </c>
+      <c r="H1501" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1501" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1501" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1501" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1501" s="4" t="s">
+        <v>1728</v>
+      </c>
+      <c r="M1501" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1502" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1502" s="4">
+        <v>509</v>
+      </c>
+      <c r="B1502" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1502" s="8">
+        <v>119191</v>
+      </c>
+      <c r="D1502" s="10">
+        <v>46255.64077391204</v>
+      </c>
+      <c r="E1502" s="8" t="s">
+        <v>1508</v>
+      </c>
+      <c r="F1502" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1502" s="8" t="s">
+        <v>1679</v>
+      </c>
+      <c r="H1502" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1502" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1502" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1502" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1502" s="4" t="s">
+        <v>1729</v>
+      </c>
+      <c r="M1502" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1503" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1503" s="4">
+        <v>510</v>
+      </c>
+      <c r="B1503" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1503" s="8">
+        <v>115367</v>
+      </c>
+      <c r="D1503" s="10">
+        <v>46255.645053310189</v>
+      </c>
+      <c r="E1503" s="8" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1503" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1503" s="8" t="s">
+        <v>1680</v>
+      </c>
+      <c r="H1503" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1503" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1503" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1503" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1503" s="4" t="s">
+        <v>1730</v>
+      </c>
+      <c r="M1503" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1504" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1504" s="4">
+        <v>511</v>
+      </c>
+      <c r="B1504" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1504" s="8">
+        <v>117177</v>
+      </c>
+      <c r="D1504" s="10">
+        <v>46255.649247083333</v>
+      </c>
+      <c r="E1504" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1504" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1504" s="8" t="s">
+        <v>1681</v>
+      </c>
+      <c r="H1504" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1504" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1504" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1504" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1504" s="4" t="s">
+        <v>1731</v>
+      </c>
+      <c r="M1504" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1505" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1505" s="4">
+        <v>512</v>
+      </c>
+      <c r="B1505" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1505" s="8">
+        <v>123664</v>
+      </c>
+      <c r="D1505" s="10">
+        <v>46255.673882916657</v>
+      </c>
+      <c r="E1505" s="8" t="s">
+        <v>1610</v>
+      </c>
+      <c r="F1505" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1505" s="8" t="s">
+        <v>1682</v>
+      </c>
+      <c r="H1505" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1505" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1505" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1505" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1505" s="4" t="s">
+        <v>1732</v>
+      </c>
+      <c r="M1505" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1506" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1506" s="4">
+        <v>513</v>
+      </c>
+      <c r="B1506" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1506" s="8">
+        <v>105564</v>
+      </c>
+      <c r="D1506" s="10">
+        <v>46255.75913697917</v>
+      </c>
+      <c r="E1506" s="8" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F1506" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1506" s="8" t="s">
+        <v>1683</v>
+      </c>
+      <c r="H1506" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1506" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1506" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1506" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1506" s="4" t="s">
+        <v>1733</v>
+      </c>
+      <c r="M1506" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1507" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1507" s="4">
+        <v>514</v>
+      </c>
+      <c r="B1507" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1507" s="8">
+        <v>118216</v>
+      </c>
+      <c r="D1507" s="10">
+        <v>46255.769036481477</v>
+      </c>
+      <c r="E1507" s="8" t="s">
+        <v>1508</v>
+      </c>
+      <c r="F1507" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1507" s="8" t="s">
+        <v>1684</v>
+      </c>
+      <c r="H1507" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1507" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1507" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1507" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1507" s="4" t="s">
+        <v>1734</v>
+      </c>
+      <c r="M1507" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1508" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1508" s="4">
+        <v>515</v>
+      </c>
+      <c r="B1508" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1508" s="8">
+        <v>117952</v>
+      </c>
+      <c r="D1508" s="10">
+        <v>46255.784961990743</v>
+      </c>
+      <c r="E1508" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1508" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1508" s="8" t="s">
+        <v>1685</v>
+      </c>
+      <c r="H1508" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1508" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1508" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1508" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1508" s="4" t="s">
+        <v>1735</v>
+      </c>
+      <c r="M1508" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1509" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1509" s="4">
+        <v>516</v>
+      </c>
+      <c r="B1509" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1509" s="8">
+        <v>119350</v>
+      </c>
+      <c r="D1509" s="10">
+        <v>46256.386197175932</v>
+      </c>
+      <c r="E1509" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="F1509" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1509" s="8" t="s">
+        <v>1686</v>
+      </c>
+      <c r="H1509" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1509" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1509" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1509" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1509" s="4" t="s">
+        <v>1736</v>
+      </c>
+      <c r="M1509" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1510" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1510" s="4">
+        <v>517</v>
+      </c>
+      <c r="B1510" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1510" s="8">
+        <v>118904</v>
+      </c>
+      <c r="D1510" s="10">
+        <v>46256.60289790509</v>
+      </c>
+      <c r="E1510" s="8" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1510" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1510" s="8" t="s">
+        <v>1687</v>
+      </c>
+      <c r="H1510" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1510" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1510" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1510" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1510" s="4" t="s">
+        <v>1737</v>
+      </c>
+      <c r="M1510" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1511" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1511" s="4">
+        <v>518</v>
+      </c>
+      <c r="B1511" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1511" s="8">
+        <v>125265</v>
+      </c>
+      <c r="D1511" s="10">
+        <v>46256.629825138887</v>
+      </c>
+      <c r="E1511" s="8" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F1511" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1511" s="8" t="s">
+        <v>1688</v>
+      </c>
+      <c r="H1511" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1511" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1511" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1511" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1511" s="4" t="s">
+        <v>1738</v>
+      </c>
+      <c r="M1511" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1512" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1512" s="4">
+        <v>519</v>
+      </c>
+      <c r="B1512" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1512" s="8">
+        <v>127160</v>
+      </c>
+      <c r="D1512" s="10">
+        <v>46256.844575266201</v>
+      </c>
+      <c r="E1512" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1512" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1512" s="8" t="s">
+        <v>1689</v>
+      </c>
+      <c r="H1512" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1512" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1512" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1512" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1512" s="4" t="s">
+        <v>1739</v>
+      </c>
+      <c r="M1512" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1513" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1513" s="4">
+        <v>520</v>
+      </c>
+      <c r="B1513" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C1513" s="8">
+        <v>114540</v>
+      </c>
+      <c r="D1513" s="10">
+        <v>46257.211157604157</v>
+      </c>
+      <c r="E1513" s="8" t="s">
+        <v>1244</v>
+      </c>
+      <c r="F1513" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1513" s="8" t="s">
+        <v>1690</v>
+      </c>
+      <c r="H1513" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1513" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1513" s="4" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1513" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1513" s="4" t="s">
+        <v>1740</v>
+      </c>
+      <c r="M1513" s="4" t="s">
+        <v>1692</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 28/08/2026 11:43:06,66
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="907" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD3975A2-3AB1-4DF1-A5DB-71AE92081015}"/>
+  <xr:revisionPtr revIDLastSave="964" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56139A71-272B-4544-BA3D-179BB2D66D37}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="1920" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12218" uniqueCount="1741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12338" uniqueCount="1765">
   <si>
     <t>ID</t>
   </si>
@@ -5463,11 +5463,104 @@
   <si>
     <t>atendimento não durou 5 minutos, só cola selo</t>
   </si>
+  <si>
+    <t>Porque o tecnico não se preocupou em resolver algumas das nossas reclamações.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ .
+Porque o serviço prestado esta muito aquem do foi vendido no contrato. O aparelho apresentou problema fiz o chamado para assistencia técnica e desde a primeira visita o técnico solicitou a troca do aparelho, já retornou mais uma vez e até a presente data sigo com o aparelho operando com defeito. Equipamento oferecido em conbtrato com água gelada e gaseificada, hoje estou bebendo agua natural. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estou com um problema no meu purificador, recorrente,a quase um ano! Sou cliente a mais de cinco anos, já solicitei a troca do mesmo e não fui atendido!!!!
+</t>
+  </si>
+  <si>
+    <t>Solicitamos reparo em um purificador que estava vazando, depois de demorar muito foi efetuada a substituição. Todavia, no mesmo dia identificamos que o equipamento "novo" não estava gelando e solicitamos o reparo. Faz mais de um mês que não temos água gelada. Não é admissível, visto que o propósito de se locar um equipamento é ter tranquilidade nas manuteções periódicas e emergenciais. Tinha-mos dois contratos e um já cancelamos. Em breve cancelaremos o outro caso o serviço continue precário.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque o serviço de vocês continua péssimo. Agendei para o período da tarde, o técnico veio de manhã. A sorte é que a minha filha ainda nao tinha saído. 
+</t>
+  </si>
+  <si>
+    <t>TIVEMOS QUE CHAMAR O TECNICO 2 VEZES E MESMO ASSIM O FILTRO CONTINUA VAZANDO.</t>
+  </si>
+  <si>
+    <t>Eu agendei para o período da tarde e o técnico veio por volta das 11h da manhã.
+Isto demonstra a desorganização da empresa. Dois agendamentos não atendidos e um terceiro atendido fora do horário agendado.</t>
+  </si>
+  <si>
+    <t>O tecnico nem veio! Já reclamei duas vezes que o filtro pinga, inclusive com videos enviados e depois de um dia para de pingar. o técnico veio e não fez nada.</t>
+  </si>
+  <si>
+    <t>A técnica chegou às 15:40h,  partir do que copio aqui a seguir, porque será que minha avaliação foi essa?????
+[11:10, 11/08/2026] Ju: Certo, então para confirmar você deseja uma visita técnica no seguinte período:
+Dia da Visita: Segunda-feira
+Data da Visita: 24/08/2026
+Período da Visita: Manhã - Entre 08h e 13h
+É isso mesmo?
+Por gentileza, me responda com sim ou não
+[11:10, 11/08/2026] Ju: ✅ A visita técnica foi agendada com sucesso. 
+📝 É importante que você anote o número da ordem de serviço:  00274421 e a sua senha de atendimento: 182295. 
+Outras informações importantes: 
+Nesta visita, o elemento filtrante somente será trocado se o teste de qualidade da água for reprovado pelo técnico.
+É necessário que alguém maior de 18 anos esteja no local para acompanhar o técnico no momento da visita.
+💡 Ah, e caso você não precise mais da visita do técnico ou quiser reagendá-la, entre em contato conosco. 😉</t>
+  </si>
+  <si>
+    <t>muitissimo caro</t>
+  </si>
+  <si>
+    <t>entrei em contato hoje com vocês, ninguem a apareceu aqui e no sistema consta que foi visitado sim. porem, nem no filtro foi trocado a etiqueta de validade da manutenção</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ficou atrasada a visita, saiu do conserto com gosto de metal ainda no purificador. </t>
+  </si>
+  <si>
+    <t>técnico não resolveu as reclamações</t>
+  </si>
+  <si>
+    <t>troca solicitada, 2 visitas, defeito persiste</t>
+  </si>
+  <si>
+    <t>problema recorrente há quase um ano</t>
+  </si>
+  <si>
+    <t>equipamento novo não gela + demora</t>
+  </si>
+  <si>
+    <t>agendou tarde, técnico veio de manhã</t>
+  </si>
+  <si>
+    <t>2 visitas e filtro continua vazando</t>
+  </si>
+  <si>
+    <t>veio 11h para tarde + 2 agendamentos não atendidos</t>
+  </si>
+  <si>
+    <t>técnico veio e não fez nada, filtro pinga</t>
+  </si>
+  <si>
+    <t>agendado 8-13h, técnica chegou 15:40h</t>
+  </si>
+  <si>
+    <t>muitíssimo caro</t>
+  </si>
+  <si>
+    <t>ninguém apareceu, sistema consta visitado</t>
+  </si>
+  <si>
+    <t>gosto de metal após conserto + visita atrasada</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -5550,7 +5643,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5580,6 +5673,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -5884,7 +5980,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="8">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="10">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -5906,7 +6002,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1513"/>
+  <dimension ref="A1:M1525"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -59171,6 +59267,498 @@
         <v>1692</v>
       </c>
     </row>
+    <row r="1514" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1514" s="4">
+        <v>521</v>
+      </c>
+      <c r="B1514" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1514" s="8">
+        <v>114326</v>
+      </c>
+      <c r="D1514" s="11">
+        <v>46258.523561828697</v>
+      </c>
+      <c r="E1514" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1514" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1514" s="8" t="s">
+        <v>1741</v>
+      </c>
+      <c r="H1514" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1514" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1514" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1514" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1514" s="4" t="s">
+        <v>1753</v>
+      </c>
+      <c r="M1514" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1515" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1515" s="4">
+        <v>522</v>
+      </c>
+      <c r="B1515" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1515" s="8">
+        <v>124580</v>
+      </c>
+      <c r="D1515" s="11">
+        <v>46258.779456412027</v>
+      </c>
+      <c r="E1515" s="8" t="s">
+        <v>1580</v>
+      </c>
+      <c r="F1515" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1515" s="8" t="s">
+        <v>1742</v>
+      </c>
+      <c r="H1515" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1515" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1515" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1515" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1515" s="4" t="s">
+        <v>1754</v>
+      </c>
+      <c r="M1515" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1516" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1516" s="4">
+        <v>523</v>
+      </c>
+      <c r="B1516" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1516" s="8">
+        <v>129091</v>
+      </c>
+      <c r="D1516" s="11">
+        <v>46258.838097372682</v>
+      </c>
+      <c r="E1516" s="8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="F1516" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1516" s="8" t="s">
+        <v>1743</v>
+      </c>
+      <c r="H1516" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1516" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1516" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1516" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1516" s="4" t="s">
+        <v>1755</v>
+      </c>
+      <c r="M1516" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1517" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1517" s="4">
+        <v>524</v>
+      </c>
+      <c r="B1517" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1517" s="8">
+        <v>127403</v>
+      </c>
+      <c r="D1517" s="11">
+        <v>46259.595003784721</v>
+      </c>
+      <c r="E1517" s="8" t="s">
+        <v>1612</v>
+      </c>
+      <c r="F1517" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1517" s="8" t="s">
+        <v>1744</v>
+      </c>
+      <c r="H1517" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1517" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1517" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1517" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1517" s="4" t="s">
+        <v>1756</v>
+      </c>
+      <c r="M1517" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1518" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1518" s="4">
+        <v>525</v>
+      </c>
+      <c r="B1518" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1518" s="8">
+        <v>119438</v>
+      </c>
+      <c r="D1518" s="11">
+        <v>46259.967046863429</v>
+      </c>
+      <c r="E1518" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1518" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1518" s="8" t="s">
+        <v>1745</v>
+      </c>
+      <c r="H1518" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1518" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1518" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1518" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1518" s="4" t="s">
+        <v>1757</v>
+      </c>
+      <c r="M1518" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1519" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1519" s="4">
+        <v>526</v>
+      </c>
+      <c r="B1519" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1519" s="8">
+        <v>125139</v>
+      </c>
+      <c r="D1519" s="11">
+        <v>46260.656516157411</v>
+      </c>
+      <c r="E1519" s="8" t="s">
+        <v>1416</v>
+      </c>
+      <c r="F1519" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1519" s="8" t="s">
+        <v>1746</v>
+      </c>
+      <c r="H1519" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1519" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1519" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1519" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1519" s="4" t="s">
+        <v>1758</v>
+      </c>
+      <c r="M1519" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1520" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1520" s="4">
+        <v>527</v>
+      </c>
+      <c r="B1520" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1520" s="8">
+        <v>124378</v>
+      </c>
+      <c r="D1520" s="11">
+        <v>46260.664259895842</v>
+      </c>
+      <c r="E1520" s="8" t="s">
+        <v>1252</v>
+      </c>
+      <c r="F1520" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1520" s="8" t="s">
+        <v>1747</v>
+      </c>
+      <c r="H1520" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1520" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1520" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1520" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1520" s="4" t="s">
+        <v>1759</v>
+      </c>
+      <c r="M1520" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1521" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1521" s="4">
+        <v>528</v>
+      </c>
+      <c r="B1521" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1521" s="8">
+        <v>110980</v>
+      </c>
+      <c r="D1521" s="11">
+        <v>46260.670854861113</v>
+      </c>
+      <c r="E1521" s="8" t="s">
+        <v>1610</v>
+      </c>
+      <c r="F1521" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1521" s="8" t="s">
+        <v>1748</v>
+      </c>
+      <c r="H1521" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1521" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1521" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1521" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1521" s="4" t="s">
+        <v>1760</v>
+      </c>
+      <c r="M1521" s="4" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1522" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1522" s="4">
+        <v>529</v>
+      </c>
+      <c r="B1522" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1522" s="8">
+        <v>120498</v>
+      </c>
+      <c r="D1522" s="11">
+        <v>46260.698743657413</v>
+      </c>
+      <c r="E1522" s="8" t="s">
+        <v>1248</v>
+      </c>
+      <c r="F1522" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1522" s="8" t="s">
+        <v>1749</v>
+      </c>
+      <c r="H1522" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1522" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1522" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1522" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1522" s="4" t="s">
+        <v>1761</v>
+      </c>
+      <c r="M1522" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1523" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1523" s="4">
+        <v>530</v>
+      </c>
+      <c r="B1523" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1523" s="8">
+        <v>121901</v>
+      </c>
+      <c r="D1523" s="11">
+        <v>46260.70864798611</v>
+      </c>
+      <c r="E1523" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1523" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1523" s="8" t="s">
+        <v>1750</v>
+      </c>
+      <c r="H1523" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1523" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1523" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1523" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1523" s="4" t="s">
+        <v>1762</v>
+      </c>
+      <c r="M1523" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1524" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1524" s="4">
+        <v>531</v>
+      </c>
+      <c r="B1524" s="8" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C1524" s="8">
+        <v>126105</v>
+      </c>
+      <c r="D1524" s="11">
+        <v>46260.825613090281</v>
+      </c>
+      <c r="E1524" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="F1524" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1524" s="8" t="s">
+        <v>1751</v>
+      </c>
+      <c r="H1524" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1524" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J1524" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1524" s="8" t="s">
+        <v>1441</v>
+      </c>
+      <c r="L1524" s="4" t="s">
+        <v>1763</v>
+      </c>
+      <c r="M1524" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1525" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1525" s="4">
+        <v>532</v>
+      </c>
+      <c r="B1525" s="8" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C1525" s="8">
+        <v>21536</v>
+      </c>
+      <c r="D1525" s="11">
+        <v>46260.895230983799</v>
+      </c>
+      <c r="E1525" s="8" t="s">
+        <v>1653</v>
+      </c>
+      <c r="F1525" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1525" s="8" t="s">
+        <v>1752</v>
+      </c>
+      <c r="H1525" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1525" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1525" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="K1525" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="L1525" s="4" t="s">
+        <v>1764</v>
+      </c>
+      <c r="M1525" s="4" t="s">
+        <v>1692</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 03/09/2026 11:27:38,12
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1092" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FBCB330-930F-4737-9BDD-71485F7A6B04}"/>
+  <xr:revisionPtr revIDLastSave="1113" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3901553-C985-4D5A-B2FD-302E43027E44}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-13620" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12536" uniqueCount="1799">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12572" uniqueCount="1805">
   <si>
     <t>ID</t>
   </si>
@@ -5660,6 +5660,24 @@
   </si>
   <si>
     <t>mensagens do WhatsApp não são cumpridas</t>
+  </si>
+  <si>
+    <t>02/09/2026</t>
+  </si>
+  <si>
+    <t>03/09/2026</t>
+  </si>
+  <si>
+    <t>Ele veio para fazer a manutencao preventiva dentre ela a troca do filtro e depois de 6 meses disse que nao era necessario. Foi embora sem higienizar o aparelho ou trocar o filtro. Para que manutencao de 6 em 6 meses se nem o filtro foi trocado?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A pior possível, sou cliente há 14 anos e nunca me senti tão mal atendido, solicitei uma visita, pois meu filtro está fazendo um barulho insuportável, o técnico confirmou o problema, ao enviar um vídeo para central a atendente disse que não havia problema algum no filtro na minha cara e do técnico, reintero que o técnico foi ótimo, sabia o que estava fazendo e falando, mas uma funcionária de dentro de um escritório no ar condicionado fala na minha cara que meu filtro não tem problema nenhum. Vou cancelar! </t>
+  </si>
+  <si>
+    <t>O meu aparelho foi instalado a menos de uma semana e já apresentou defeito, manutenção só acontecerá após 2 dias.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meu filtro não tem nem dois meses e já deu problema. Queria que mudassem para um novo </t>
   </si>
 </sst>
 </file>
@@ -5751,7 +5769,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5785,6 +5803,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6127,7 +6148,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1543"/>
+  <dimension ref="A1:M1547"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -60568,6 +60589,134 @@
         <v>1685</v>
       </c>
     </row>
+    <row r="1544" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1544" s="4" t="s">
+        <v>1406</v>
+      </c>
+      <c r="C1544" s="4">
+        <v>116728</v>
+      </c>
+      <c r="D1544" s="2" t="s">
+        <v>1799</v>
+      </c>
+      <c r="E1544" s="4" t="s">
+        <v>1424</v>
+      </c>
+      <c r="F1544" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1544" s="4" t="s">
+        <v>1801</v>
+      </c>
+      <c r="H1544" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1544" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1544" s="4" t="s">
+        <v>1399</v>
+      </c>
+      <c r="K1544" s="4" t="s">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="1545" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1545" s="4" t="s">
+        <v>1302</v>
+      </c>
+      <c r="C1545" s="4">
+        <v>134157</v>
+      </c>
+      <c r="D1545" s="2" t="s">
+        <v>1799</v>
+      </c>
+      <c r="E1545" s="4" t="s">
+        <v>1481</v>
+      </c>
+      <c r="F1545" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1545" s="4" t="s">
+        <v>1802</v>
+      </c>
+      <c r="H1545" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1545" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1545" s="4" t="s">
+        <v>1399</v>
+      </c>
+      <c r="K1545" s="4" t="s">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="1546" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1546" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1546" s="4">
+        <v>132917</v>
+      </c>
+      <c r="D1546" s="2" t="s">
+        <v>1800</v>
+      </c>
+      <c r="E1546" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="F1546" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1546" s="4" t="s">
+        <v>1803</v>
+      </c>
+      <c r="H1546" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1546" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1546" s="4" t="s">
+        <v>1399</v>
+      </c>
+      <c r="K1546" s="4" t="s">
+        <v>1436</v>
+      </c>
+    </row>
+    <row r="1547" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1547" s="4" t="s">
+        <v>1302</v>
+      </c>
+      <c r="C1547" s="4">
+        <v>131662</v>
+      </c>
+      <c r="D1547" s="2" t="s">
+        <v>1800</v>
+      </c>
+      <c r="E1547" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1547" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1547" s="4" t="s">
+        <v>1804</v>
+      </c>
+      <c r="H1547" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1547" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1547" s="4" t="s">
+        <v>1399</v>
+      </c>
+      <c r="K1547" s="4" t="s">
+        <v>1434</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 03/09/2026 14:57:04,64
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1113" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3901553-C985-4D5A-B2FD-302E43027E44}"/>
+  <xr:revisionPtr revIDLastSave="1134" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A18CB5A-E8A8-4F7E-B776-32BA5B3BAB2C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1451</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1547</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -5769,7 +5769,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5806,6 +5806,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -55730,7 +55733,7 @@
         <v>1434</v>
       </c>
     </row>
-    <row r="1417" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1417" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A1417" s="4">
         <v>421</v>
       </c>
@@ -55749,7 +55752,7 @@
       <c r="F1417" s="4" t="s">
         <v>1458</v>
       </c>
-      <c r="G1417" s="4" t="s">
+      <c r="G1417" s="5" t="s">
         <v>1585</v>
       </c>
       <c r="H1417" s="4" t="s">
@@ -56535,7 +56538,7 @@
         <v>1434</v>
       </c>
     </row>
-    <row r="1440" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1440" spans="1:11" ht="210" x14ac:dyDescent="0.25">
       <c r="A1440" s="4">
         <v>444</v>
       </c>
@@ -56554,7 +56557,7 @@
       <c r="F1440" t="s">
         <v>16</v>
       </c>
-      <c r="G1440" s="8" t="s">
+      <c r="G1440" s="13" t="s">
         <v>1609</v>
       </c>
       <c r="H1440" s="4" t="s">
@@ -56605,7 +56608,7 @@
         <v>1434</v>
       </c>
     </row>
-    <row r="1442" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1442" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A1442" s="4">
         <v>447</v>
       </c>
@@ -56624,7 +56627,7 @@
       <c r="F1442" t="s">
         <v>16</v>
       </c>
-      <c r="G1442" s="8" t="s">
+      <c r="G1442" s="13" t="s">
         <v>1611</v>
       </c>
       <c r="H1442" s="4" t="s">
@@ -57568,7 +57571,7 @@
         <v>1687</v>
       </c>
     </row>
-    <row r="1469" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1469" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A1469" s="4">
         <v>476</v>
       </c>
@@ -57587,14 +57590,14 @@
       <c r="F1469" t="s">
         <v>16</v>
       </c>
-      <c r="G1469" s="8" t="s">
+      <c r="G1469" s="13" t="s">
         <v>1640</v>
       </c>
       <c r="H1469" s="4" t="s">
-        <v>80</v>
+        <v>1528</v>
       </c>
       <c r="I1469" s="4" t="s">
-        <v>81</v>
+        <v>1555</v>
       </c>
       <c r="J1469" s="4" t="s">
         <v>1399</v>
@@ -57960,10 +57963,10 @@
         <v>1631</v>
       </c>
       <c r="H1478" s="4" t="s">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="I1478" s="4" t="s">
-        <v>414</v>
+        <v>26</v>
       </c>
       <c r="J1478" s="4" t="s">
         <v>1399</v>
@@ -58329,10 +58332,10 @@
         <v>1658</v>
       </c>
       <c r="H1487" s="4" t="s">
-        <v>80</v>
+        <v>1528</v>
       </c>
       <c r="I1487" s="4" t="s">
-        <v>81</v>
+        <v>1555</v>
       </c>
       <c r="J1487" s="4" t="s">
         <v>1399</v>

</xml_diff>